<commit_message>
update column AC sprint 1.1
</commit_message>
<xml_diff>
--- a/sprint_1/1_business_analysis/deliverables/AC.xlsx
+++ b/sprint_1/1_business_analysis/deliverables/AC.xlsx
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="253" uniqueCount="105">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="278" uniqueCount="114">
   <si>
     <t>STT</t>
   </si>
@@ -196,6 +196,9 @@
     <t>AC234 – Smart City Chatbot Questions (SNI ISO 37122:2019)</t>
   </si>
   <si>
+    <t>Technical Evaluate</t>
+  </si>
+  <si>
     <t>Câu hỏi</t>
   </si>
   <si>
@@ -211,6 +214,12 @@
     <t>Nhóm nghiệp vụ/dữ liệu</t>
   </si>
   <si>
+    <t>Cách tính</t>
+  </si>
+  <si>
+    <t>Nguồn dữ liệu</t>
+  </si>
+  <si>
     <t xml:space="preserve">PHẦN 1: CÂU HỎI CHO CƯ DÂN (RESIDENT) </t>
   </si>
   <si>
@@ -298,7 +307,7 @@
     <t>Danh sách các thiết bị thông minh lắp đặt ngoài trời bị hư hỏng</t>
   </si>
   <si>
-    <t>Phát thông báo dọn rác cho nhân viên khi có thùng rác đầy</t>
+    <t>Danh sách các thùng rác đang đầy</t>
   </si>
   <si>
     <t>Percentage of the city population that has a door-to-door garbage collection with an individual monitoring of household waste quantities + Percentage of public garbage bins that are sensor-enabled public garbage bins</t>
@@ -331,6 +340,12 @@
     <t>Tỉ lệ khả năng lưu trữ của mạng lưới điện hiện tại so với tổng lượng điện tiêu thụ</t>
   </si>
   <si>
+    <t>Danh sách các nguồn cấp điện bị quá tải</t>
+  </si>
+  <si>
+    <t>Danh sách các hệ thống cấp nước bị hỏng</t>
+  </si>
+  <si>
     <t>Số lượng đèn tín hiệu giao thông thông minh hiện tại, lọc theo trạng thái (hoạt động bình thường/hư hỏng)</t>
   </si>
   <si>
@@ -344,6 +359,18 @@
   </si>
   <si>
     <t>G</t>
+  </si>
+  <si>
+    <t>PHẦN 2: CÂU HỎI BỔ SUNG THÊM KHÔNG MAPPING VỚI ISO 37122 INDICATOR</t>
+  </si>
+  <si>
+    <t>Danh sách các thiết bị ra/vào tòa nhà không hoạt động/bị hỏng</t>
+  </si>
+  <si>
+    <t>Lọc theo trạng thái / khu vực</t>
+  </si>
+  <si>
+    <t>Danh sách các thang máy đang trong trạng thái không hoạt động/hư hỏng/bảo trì</t>
   </si>
 </sst>
 </file>
@@ -528,12 +555,42 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="33">
+  <fills count="38">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.6"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.6"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="8" tint="0.4"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.8"/>
+        <bgColor indexed="64"/>
+      </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
@@ -728,21 +785,6 @@
       <right/>
       <top/>
       <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
       <diagonal/>
     </border>
     <border>
@@ -771,6 +813,21 @@
     </border>
     <border>
       <left/>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
       <right style="thin">
         <color auto="1"/>
       </right>
@@ -943,7 +1000,7 @@
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="8" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="8" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -967,16 +1024,16 @@
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="3" borderId="11" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="4" borderId="12" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="4" borderId="11" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="5" borderId="13" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="12" fillId="8" borderId="11" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="9" borderId="12" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="9" borderId="11" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="10" borderId="13" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="14" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
@@ -985,138 +1042,168 @@
     <xf numFmtId="0" fontId="17" fillId="0" borderId="15" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="18" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="22" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="21" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="22" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="21" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="22" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="21" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="22" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="21" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="21" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="22" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="22" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="36" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="37" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="30">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1674,26 +1761,26 @@
   </cols>
   <sheetData>
     <row r="1" ht="17.4" spans="1:8">
-      <c r="A1" s="14" t="s">
+      <c r="A1" s="24" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="14" t="s">
+      <c r="B1" s="24" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="14"/>
-      <c r="D1" s="14" t="s">
+      <c r="C1" s="24"/>
+      <c r="D1" s="24" t="s">
         <v>2</v>
       </c>
-      <c r="E1" s="14" t="s">
+      <c r="E1" s="24" t="s">
         <v>3</v>
       </c>
-      <c r="F1" s="15" t="s">
+      <c r="F1" s="25" t="s">
         <v>4</v>
       </c>
-      <c r="G1" s="15" t="s">
+      <c r="G1" s="25" t="s">
         <v>5</v>
       </c>
-      <c r="H1" s="15" t="s">
+      <c r="H1" s="25" t="s">
         <v>6</v>
       </c>
     </row>
@@ -1716,8 +1803,8 @@
       <c r="F2" s="12">
         <v>7.1</v>
       </c>
-      <c r="G2" s="16"/>
-      <c r="H2" s="5"/>
+      <c r="G2" s="26"/>
+      <c r="H2" s="21"/>
     </row>
     <row r="3" ht="36" spans="1:8">
       <c r="A3" s="9"/>
@@ -1734,8 +1821,8 @@
       <c r="F3" s="12">
         <v>19.8</v>
       </c>
-      <c r="G3" s="16"/>
-      <c r="H3" s="5"/>
+      <c r="G3" s="26"/>
+      <c r="H3" s="21"/>
     </row>
     <row r="4" ht="36" spans="1:8">
       <c r="A4" s="9"/>
@@ -1752,8 +1839,8 @@
       <c r="F4" s="12">
         <v>12.1</v>
       </c>
-      <c r="G4" s="16"/>
-      <c r="H4" s="5"/>
+      <c r="G4" s="26"/>
+      <c r="H4" s="21"/>
     </row>
     <row r="5" ht="36" spans="1:8">
       <c r="A5" s="9"/>
@@ -1768,8 +1855,8 @@
       <c r="F5" s="12">
         <v>12.2</v>
       </c>
-      <c r="G5" s="16"/>
-      <c r="H5" s="5"/>
+      <c r="G5" s="26"/>
+      <c r="H5" s="21"/>
     </row>
     <row r="6" ht="36" spans="1:8">
       <c r="A6" s="9"/>
@@ -1784,8 +1871,8 @@
       <c r="F6" s="12">
         <v>8.3</v>
       </c>
-      <c r="G6" s="16"/>
-      <c r="H6" s="5"/>
+      <c r="G6" s="26"/>
+      <c r="H6" s="21"/>
     </row>
     <row r="7" ht="36" spans="1:8">
       <c r="A7" s="9"/>
@@ -1802,8 +1889,8 @@
       <c r="F7" s="12">
         <v>7.6</v>
       </c>
-      <c r="G7" s="16"/>
-      <c r="H7" s="5"/>
+      <c r="G7" s="26"/>
+      <c r="H7" s="21"/>
     </row>
     <row r="8" ht="36" spans="1:8">
       <c r="A8" s="9"/>
@@ -1818,8 +1905,8 @@
       <c r="F8" s="12">
         <v>7.7</v>
       </c>
-      <c r="G8" s="16"/>
-      <c r="H8" s="5"/>
+      <c r="G8" s="26"/>
+      <c r="H8" s="21"/>
     </row>
     <row r="9" ht="54" spans="1:8">
       <c r="A9" s="9">
@@ -1840,8 +1927,8 @@
       <c r="F9" s="12">
         <v>8.2</v>
       </c>
-      <c r="G9" s="16"/>
-      <c r="H9" s="5"/>
+      <c r="G9" s="26"/>
+      <c r="H9" s="21"/>
     </row>
     <row r="10" ht="54" spans="1:8">
       <c r="A10" s="9"/>
@@ -1858,8 +1945,8 @@
       <c r="F10" s="12">
         <v>23.2</v>
       </c>
-      <c r="G10" s="16"/>
-      <c r="H10" s="5"/>
+      <c r="G10" s="26"/>
+      <c r="H10" s="21"/>
     </row>
     <row r="11" ht="72" spans="1:8">
       <c r="A11" s="9"/>
@@ -1876,8 +1963,8 @@
       <c r="F11" s="12">
         <v>16.2</v>
       </c>
-      <c r="G11" s="16"/>
-      <c r="H11" s="5"/>
+      <c r="G11" s="26"/>
+      <c r="H11" s="21"/>
     </row>
     <row r="12" ht="36" spans="1:8">
       <c r="A12" s="9"/>
@@ -1892,8 +1979,8 @@
       <c r="F12" s="12">
         <v>16.5</v>
       </c>
-      <c r="G12" s="16"/>
-      <c r="H12" s="5"/>
+      <c r="G12" s="26"/>
+      <c r="H12" s="21"/>
     </row>
     <row r="13" ht="36" spans="1:8">
       <c r="A13" s="9"/>
@@ -1908,11 +1995,11 @@
       <c r="F13" s="12">
         <v>16.1</v>
       </c>
-      <c r="G13" s="16"/>
-      <c r="H13" s="5"/>
+      <c r="G13" s="26"/>
+      <c r="H13" s="21"/>
     </row>
     <row r="14" ht="54" spans="1:8">
-      <c r="A14" s="17">
+      <c r="A14" s="27">
         <v>3</v>
       </c>
       <c r="B14" s="10" t="s">
@@ -1928,11 +2015,11 @@
       <c r="F14" s="12">
         <v>7.4</v>
       </c>
-      <c r="G14" s="16"/>
-      <c r="H14" s="5"/>
+      <c r="G14" s="26"/>
+      <c r="H14" s="21"/>
     </row>
     <row r="15" ht="36" spans="1:8">
-      <c r="A15" s="18"/>
+      <c r="A15" s="28"/>
       <c r="B15" s="10"/>
       <c r="C15" s="10"/>
       <c r="D15" s="10" t="s">
@@ -1944,11 +2031,11 @@
       <c r="F15" s="12">
         <v>7.5</v>
       </c>
-      <c r="G15" s="16"/>
-      <c r="H15" s="5"/>
+      <c r="G15" s="26"/>
+      <c r="H15" s="21"/>
     </row>
     <row r="16" ht="36" spans="1:8">
-      <c r="A16" s="17">
+      <c r="A16" s="27">
         <v>4</v>
       </c>
       <c r="B16" s="10" t="s">
@@ -1964,11 +2051,11 @@
       <c r="F16" s="12">
         <v>19.3</v>
       </c>
-      <c r="G16" s="16"/>
-      <c r="H16" s="5"/>
+      <c r="G16" s="26"/>
+      <c r="H16" s="21"/>
     </row>
     <row r="17" ht="36" spans="1:8">
-      <c r="A17" s="19"/>
+      <c r="A17" s="29"/>
       <c r="B17" s="10"/>
       <c r="C17" s="10"/>
       <c r="D17" s="10" t="s">
@@ -1980,11 +2067,11 @@
       <c r="F17" s="12">
         <v>19.9</v>
       </c>
-      <c r="G17" s="16"/>
-      <c r="H17" s="5"/>
+      <c r="G17" s="26"/>
+      <c r="H17" s="21"/>
     </row>
     <row r="18" ht="36" spans="1:8">
-      <c r="A18" s="18"/>
+      <c r="A18" s="28"/>
       <c r="B18" s="10"/>
       <c r="C18" s="10"/>
       <c r="D18" s="10" t="s">
@@ -1996,8 +2083,8 @@
       <c r="F18" s="12">
         <v>19.1</v>
       </c>
-      <c r="G18" s="16"/>
-      <c r="H18" s="5"/>
+      <c r="G18" s="26"/>
+      <c r="H18" s="21"/>
     </row>
     <row r="19" ht="36" spans="1:8">
       <c r="A19" s="9">
@@ -2016,8 +2103,8 @@
       <c r="F19" s="12">
         <v>15.1</v>
       </c>
-      <c r="G19" s="16"/>
-      <c r="H19" s="5"/>
+      <c r="G19" s="26"/>
+      <c r="H19" s="21"/>
     </row>
     <row r="20" ht="18" spans="1:8">
       <c r="A20" s="9">
@@ -2034,8 +2121,8 @@
       </c>
       <c r="E20" s="10"/>
       <c r="F20" s="12"/>
-      <c r="G20" s="16"/>
-      <c r="H20" s="5"/>
+      <c r="G20" s="26"/>
+      <c r="H20" s="21"/>
     </row>
     <row r="21" ht="18" spans="1:8">
       <c r="A21" s="9"/>
@@ -2048,8 +2135,8 @@
       </c>
       <c r="E21" s="10"/>
       <c r="F21" s="12"/>
-      <c r="G21" s="16"/>
-      <c r="H21" s="5"/>
+      <c r="G21" s="26"/>
+      <c r="H21" s="21"/>
     </row>
     <row r="22" ht="18" spans="1:8">
       <c r="A22" s="9"/>
@@ -2062,8 +2149,8 @@
       </c>
       <c r="E22" s="10"/>
       <c r="F22" s="12"/>
-      <c r="G22" s="16"/>
-      <c r="H22" s="5"/>
+      <c r="G22" s="26"/>
+      <c r="H22" s="21"/>
     </row>
     <row r="23" ht="18" spans="1:8">
       <c r="A23" s="9"/>
@@ -2074,8 +2161,8 @@
       </c>
       <c r="E23" s="10"/>
       <c r="F23" s="12"/>
-      <c r="G23" s="16"/>
-      <c r="H23" s="5"/>
+      <c r="G23" s="26"/>
+      <c r="H23" s="21"/>
     </row>
     <row r="24" ht="36" spans="1:8">
       <c r="A24" s="9"/>
@@ -2088,8 +2175,8 @@
       </c>
       <c r="E24" s="10"/>
       <c r="F24" s="12"/>
-      <c r="G24" s="16"/>
-      <c r="H24" s="5"/>
+      <c r="G24" s="26"/>
+      <c r="H24" s="21"/>
     </row>
   </sheetData>
   <mergeCells count="16">
@@ -2118,7 +2205,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:L33"/>
+  <dimension ref="A1:L38"/>
   <sheetFormatPr defaultColWidth="8.88888888888889" defaultRowHeight="14.4"/>
   <cols>
     <col min="1" max="1" width="7.31481481481481" customWidth="1"/>
@@ -2129,49 +2216,66 @@
     <col min="6" max="6" width="29.3333333333333" customWidth="1"/>
     <col min="7" max="7" width="11.1018518518519" style="1" customWidth="1"/>
     <col min="8" max="8" width="28.3981481481481" customWidth="1"/>
+    <col min="9" max="9" width="36.1944444444444" customWidth="1"/>
+    <col min="10" max="10" width="39.2037037037037" customWidth="1"/>
+    <col min="11" max="11" width="21.8981481481481" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="17.4" spans="1:8">
+    <row r="1" ht="17.4" spans="1:11">
       <c r="A1" s="2" t="s">
         <v>54</v>
       </c>
       <c r="B1" s="3"/>
       <c r="C1" s="3"/>
       <c r="D1" s="3"/>
-      <c r="E1" s="4"/>
+      <c r="E1" s="3"/>
       <c r="F1" s="3"/>
-      <c r="G1" s="4"/>
-      <c r="H1" s="5"/>
-    </row>
-    <row r="2" ht="17.4" spans="1:8">
-      <c r="A2" s="2" t="s">
+      <c r="G1" s="3"/>
+      <c r="H1" s="4"/>
+      <c r="I1" s="14" t="s">
+        <v>55</v>
+      </c>
+      <c r="J1" s="15"/>
+      <c r="K1" s="16"/>
+    </row>
+    <row r="2" ht="17.4" spans="1:11">
+      <c r="A2" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="2" t="s">
-        <v>55</v>
-      </c>
-      <c r="C2" s="2" t="s">
+      <c r="B2" s="5" t="s">
+        <v>56</v>
+      </c>
+      <c r="C2" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="D2" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="E2" s="2" t="s">
-        <v>56</v>
-      </c>
-      <c r="F2" s="2" t="s">
+      <c r="E2" s="5" t="s">
         <v>57</v>
       </c>
-      <c r="G2" s="2" t="s">
+      <c r="F2" s="5" t="s">
         <v>58</v>
       </c>
-      <c r="H2" s="2" t="s">
+      <c r="G2" s="5" t="s">
         <v>59</v>
       </c>
-    </row>
-    <row r="3" ht="17.4" spans="1:8">
+      <c r="H2" s="5" t="s">
+        <v>60</v>
+      </c>
+      <c r="I2" s="17" t="s">
+        <v>61</v>
+      </c>
+      <c r="J2" s="17" t="s">
+        <v>62</v>
+      </c>
+      <c r="K2" s="17" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="3" ht="17.4" spans="1:11">
       <c r="A3" s="6" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="B3" s="7"/>
       <c r="C3" s="7"/>
@@ -2180,13 +2284,16 @@
       <c r="F3" s="7"/>
       <c r="G3" s="7"/>
       <c r="H3" s="8"/>
-    </row>
-    <row r="4" ht="72" spans="1:8">
+      <c r="I3" s="18"/>
+      <c r="J3" s="19"/>
+      <c r="K3" s="20"/>
+    </row>
+    <row r="4" ht="72" spans="1:11">
       <c r="A4" s="9">
         <v>1</v>
       </c>
       <c r="B4" s="10" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
       <c r="C4" s="10" t="s">
         <v>9</v>
@@ -2198,21 +2305,24 @@
         <v>7.1</v>
       </c>
       <c r="F4" s="11" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="G4" s="9" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="H4" s="11" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="5" ht="72" spans="1:8">
+      <c r="I4" s="21"/>
+      <c r="J4" s="21"/>
+      <c r="K4" s="21"/>
+    </row>
+    <row r="5" ht="72" spans="1:11">
       <c r="A5" s="9">
         <v>2</v>
       </c>
       <c r="B5" s="11" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="C5" s="10" t="s">
         <v>9</v>
@@ -2224,21 +2334,24 @@
         <v>7.1</v>
       </c>
       <c r="F5" s="11" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="G5" s="9" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="H5" s="11" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="6" ht="72" spans="1:8">
+      <c r="I5" s="21"/>
+      <c r="J5" s="21"/>
+      <c r="K5" s="21"/>
+    </row>
+    <row r="6" ht="72" spans="1:11">
       <c r="A6" s="9">
         <v>3</v>
       </c>
       <c r="B6" s="11" t="s">
-        <v>65</v>
+        <v>68</v>
       </c>
       <c r="C6" s="10" t="s">
         <v>9</v>
@@ -2250,21 +2363,24 @@
         <v>7.1</v>
       </c>
       <c r="F6" s="11" t="s">
+        <v>69</v>
+      </c>
+      <c r="G6" s="9" t="s">
         <v>66</v>
-      </c>
-      <c r="G6" s="9" t="s">
-        <v>63</v>
       </c>
       <c r="H6" s="11" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="7" ht="72" spans="1:8">
+      <c r="I6" s="21"/>
+      <c r="J6" s="21"/>
+      <c r="K6" s="21"/>
+    </row>
+    <row r="7" ht="72" spans="1:11">
       <c r="A7" s="9">
         <v>4</v>
       </c>
       <c r="B7" s="11" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="C7" s="10" t="s">
         <v>12</v>
@@ -2276,21 +2392,24 @@
         <v>19.8</v>
       </c>
       <c r="F7" s="11" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="G7" s="9" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="H7" s="11" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="8" ht="72" spans="1:8">
+      <c r="I7" s="21"/>
+      <c r="J7" s="21"/>
+      <c r="K7" s="21"/>
+    </row>
+    <row r="8" ht="72" spans="1:11">
       <c r="A8" s="9">
         <v>5</v>
       </c>
       <c r="B8" s="11" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="C8" s="10" t="s">
         <v>12</v>
@@ -2302,21 +2421,24 @@
         <v>19.8</v>
       </c>
       <c r="F8" s="11" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="G8" s="9" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="H8" s="11" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="9" ht="54" spans="1:8">
+      <c r="I8" s="21"/>
+      <c r="J8" s="21"/>
+      <c r="K8" s="21"/>
+    </row>
+    <row r="9" ht="54" spans="1:11">
       <c r="A9" s="9">
         <v>6</v>
       </c>
       <c r="B9" s="10" t="s">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="C9" s="11" t="s">
         <v>15</v>
@@ -2328,21 +2450,24 @@
         <v>12.1</v>
       </c>
       <c r="F9" s="11" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="G9" s="9" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="H9" s="11" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="10" ht="36" spans="1:8">
+      <c r="I9" s="21"/>
+      <c r="J9" s="21"/>
+      <c r="K9" s="21"/>
+    </row>
+    <row r="10" ht="36" spans="1:11">
       <c r="A10" s="9">
         <v>7</v>
       </c>
       <c r="B10" s="10" t="s">
-        <v>71</v>
+        <v>74</v>
       </c>
       <c r="C10" s="11" t="s">
         <v>15</v>
@@ -2354,47 +2479,53 @@
         <v>12.2</v>
       </c>
       <c r="F10" s="11" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="G10" s="9" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="H10" s="11" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="11" ht="90" spans="1:8">
+      <c r="I10" s="21"/>
+      <c r="J10" s="21"/>
+      <c r="K10" s="21"/>
+    </row>
+    <row r="11" ht="90" spans="1:11">
       <c r="A11" s="9">
         <v>8</v>
       </c>
       <c r="B11" s="10" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="C11" s="11" t="s">
         <v>15</v>
       </c>
       <c r="D11" s="10" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="E11" s="12" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
       <c r="F11" s="11" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="G11" s="9" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="H11" s="11" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="12" ht="90" spans="1:8">
+      <c r="I11" s="21"/>
+      <c r="J11" s="21"/>
+      <c r="K11" s="21"/>
+    </row>
+    <row r="12" ht="90" spans="1:11">
       <c r="A12" s="9">
         <v>9</v>
       </c>
       <c r="B12" s="11" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="C12" s="10" t="s">
         <v>18</v>
@@ -2406,21 +2537,24 @@
         <v>8.3</v>
       </c>
       <c r="F12" s="11" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="G12" s="9" t="s">
-        <v>76</v>
+        <v>79</v>
       </c>
       <c r="H12" s="11" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="13" ht="90" spans="1:8">
+      <c r="I12" s="21"/>
+      <c r="J12" s="21"/>
+      <c r="K12" s="21"/>
+    </row>
+    <row r="13" ht="90" spans="1:11">
       <c r="A13" s="9">
         <v>10</v>
       </c>
       <c r="B13" s="11" t="s">
-        <v>77</v>
+        <v>80</v>
       </c>
       <c r="C13" s="10" t="s">
         <v>18</v>
@@ -2432,21 +2566,24 @@
         <v>8.3</v>
       </c>
       <c r="F13" s="11" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="G13" s="9" t="s">
-        <v>76</v>
+        <v>79</v>
       </c>
       <c r="H13" s="11" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="14" ht="72" spans="1:8">
+      <c r="I13" s="21"/>
+      <c r="J13" s="21"/>
+      <c r="K13" s="21"/>
+    </row>
+    <row r="14" ht="72" spans="1:11">
       <c r="A14" s="9">
         <v>11</v>
       </c>
       <c r="B14" s="11" t="s">
-        <v>78</v>
+        <v>81</v>
       </c>
       <c r="C14" s="10" t="s">
         <v>18</v>
@@ -2458,33 +2595,39 @@
         <v>8.2</v>
       </c>
       <c r="F14" s="11" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="G14" s="9" t="s">
-        <v>76</v>
+        <v>79</v>
       </c>
       <c r="H14" s="11" t="s">
         <v>23</v>
       </c>
-    </row>
-    <row r="15" ht="17.4" spans="1:8">
-      <c r="A15" s="6" t="s">
-        <v>79</v>
-      </c>
-      <c r="B15" s="7"/>
-      <c r="C15" s="7"/>
-      <c r="D15" s="7"/>
-      <c r="E15" s="7"/>
-      <c r="F15" s="7"/>
-      <c r="G15" s="7"/>
-      <c r="H15" s="8"/>
+      <c r="I14" s="21"/>
+      <c r="J14" s="21"/>
+      <c r="K14" s="21"/>
+    </row>
+    <row r="15" ht="17.4" spans="1:11">
+      <c r="A15" s="13" t="s">
+        <v>82</v>
+      </c>
+      <c r="B15" s="13"/>
+      <c r="C15" s="13"/>
+      <c r="D15" s="13"/>
+      <c r="E15" s="13"/>
+      <c r="F15" s="13"/>
+      <c r="G15" s="13"/>
+      <c r="H15" s="13"/>
+      <c r="I15" s="18"/>
+      <c r="J15" s="19"/>
+      <c r="K15" s="20"/>
     </row>
     <row r="16" ht="72" spans="1:12">
       <c r="A16" s="9">
         <v>12</v>
       </c>
       <c r="B16" s="11" t="s">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="C16" s="10" t="s">
         <v>9</v>
@@ -2496,24 +2639,25 @@
         <v>7.1</v>
       </c>
       <c r="F16" s="11" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="G16" s="9" t="s">
-        <v>76</v>
+        <v>79</v>
       </c>
       <c r="H16" s="11" t="s">
         <v>7</v>
       </c>
-      <c r="J16" s="13"/>
-      <c r="K16" s="13"/>
-      <c r="L16" s="13"/>
+      <c r="I16" s="21"/>
+      <c r="J16" s="22"/>
+      <c r="K16" s="22"/>
+      <c r="L16" s="23"/>
     </row>
     <row r="17" ht="72" spans="1:12">
       <c r="A17" s="9">
         <v>13</v>
       </c>
       <c r="B17" s="11" t="s">
-        <v>82</v>
+        <v>85</v>
       </c>
       <c r="C17" s="10" t="s">
         <v>9</v>
@@ -2525,24 +2669,25 @@
         <v>7.1</v>
       </c>
       <c r="F17" s="11" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="G17" s="9" t="s">
-        <v>76</v>
+        <v>79</v>
       </c>
       <c r="H17" s="11" t="s">
         <v>7</v>
       </c>
-      <c r="J17" s="13"/>
-      <c r="K17" s="13"/>
-      <c r="L17" s="13"/>
+      <c r="I17" s="21"/>
+      <c r="J17" s="22"/>
+      <c r="K17" s="22"/>
+      <c r="L17" s="23"/>
     </row>
     <row r="18" ht="72" spans="1:12">
       <c r="A18" s="9">
         <v>14</v>
       </c>
       <c r="B18" s="11" t="s">
-        <v>83</v>
+        <v>86</v>
       </c>
       <c r="C18" s="10" t="s">
         <v>9</v>
@@ -2554,24 +2699,25 @@
         <v>7.1</v>
       </c>
       <c r="F18" s="11" t="s">
-        <v>84</v>
+        <v>87</v>
       </c>
       <c r="G18" s="9" t="s">
-        <v>76</v>
+        <v>79</v>
       </c>
       <c r="H18" s="11" t="s">
         <v>7</v>
       </c>
-      <c r="J18" s="13"/>
-      <c r="K18" s="13"/>
-      <c r="L18" s="13"/>
+      <c r="I18" s="21"/>
+      <c r="J18" s="22"/>
+      <c r="K18" s="22"/>
+      <c r="L18" s="23"/>
     </row>
     <row r="19" ht="72" spans="1:12">
       <c r="A19" s="9">
         <v>15</v>
       </c>
       <c r="B19" s="11" t="s">
-        <v>85</v>
+        <v>88</v>
       </c>
       <c r="C19" s="10" t="s">
         <v>12</v>
@@ -2583,24 +2729,25 @@
         <v>19.8</v>
       </c>
       <c r="F19" s="11" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="G19" s="9" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="H19" s="11" t="s">
         <v>7</v>
       </c>
-      <c r="J19" s="13"/>
-      <c r="K19" s="13"/>
-      <c r="L19" s="13"/>
+      <c r="I19" s="21"/>
+      <c r="J19" s="22"/>
+      <c r="K19" s="22"/>
+      <c r="L19" s="23"/>
     </row>
     <row r="20" ht="72" spans="1:12">
       <c r="A20" s="9">
         <v>16</v>
       </c>
       <c r="B20" s="11" t="s">
-        <v>86</v>
+        <v>89</v>
       </c>
       <c r="C20" s="10" t="s">
         <v>12</v>
@@ -2612,53 +2759,55 @@
         <v>19.8</v>
       </c>
       <c r="F20" s="11" t="s">
-        <v>84</v>
+        <v>87</v>
       </c>
       <c r="G20" s="9" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="H20" s="11" t="s">
         <v>7</v>
       </c>
-      <c r="J20" s="13"/>
-      <c r="K20" s="13"/>
-      <c r="L20" s="13"/>
+      <c r="I20" s="21"/>
+      <c r="J20" s="22"/>
+      <c r="K20" s="22"/>
+      <c r="L20" s="23"/>
     </row>
     <row r="21" ht="90" spans="1:12">
       <c r="A21" s="9">
         <v>17</v>
       </c>
       <c r="B21" s="11" t="s">
-        <v>87</v>
+        <v>90</v>
       </c>
       <c r="C21" s="11" t="s">
         <v>15</v>
       </c>
       <c r="D21" s="10" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="E21" s="12" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
       <c r="F21" s="11" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="G21" s="9" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="H21" s="11" t="s">
         <v>7</v>
       </c>
-      <c r="J21" s="13"/>
-      <c r="K21" s="13"/>
-      <c r="L21" s="13"/>
+      <c r="I21" s="21"/>
+      <c r="J21" s="22"/>
+      <c r="K21" s="22"/>
+      <c r="L21" s="23"/>
     </row>
     <row r="22" ht="72" spans="1:12">
       <c r="A22" s="9">
         <v>18</v>
       </c>
       <c r="B22" s="11" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="C22" s="10" t="s">
         <v>18</v>
@@ -2670,53 +2819,55 @@
         <v>8.2</v>
       </c>
       <c r="F22" s="11" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="G22" s="9" t="s">
-        <v>76</v>
+        <v>79</v>
       </c>
       <c r="H22" s="11" t="s">
         <v>23</v>
       </c>
-      <c r="J22" s="13"/>
-      <c r="K22" s="13"/>
-      <c r="L22" s="13"/>
+      <c r="I22" s="21"/>
+      <c r="J22" s="22"/>
+      <c r="K22" s="22"/>
+      <c r="L22" s="23"/>
     </row>
     <row r="23" ht="180" spans="1:12">
       <c r="A23" s="9">
         <v>19</v>
       </c>
       <c r="B23" s="11" t="s">
-        <v>89</v>
+        <v>92</v>
       </c>
       <c r="C23" s="11" t="s">
         <v>30</v>
       </c>
       <c r="D23" s="10" t="s">
-        <v>90</v>
+        <v>93</v>
       </c>
       <c r="E23" s="9" t="s">
-        <v>91</v>
+        <v>94</v>
       </c>
       <c r="F23" s="11" t="s">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="G23" s="9" t="s">
-        <v>76</v>
+        <v>79</v>
       </c>
       <c r="H23" s="11" t="s">
         <v>23</v>
       </c>
-      <c r="J23" s="13"/>
-      <c r="K23" s="13"/>
-      <c r="L23" s="13"/>
+      <c r="I23" s="21"/>
+      <c r="J23" s="22"/>
+      <c r="K23" s="22"/>
+      <c r="L23" s="23"/>
     </row>
     <row r="24" ht="72" spans="1:12">
       <c r="A24" s="9">
         <v>20</v>
       </c>
       <c r="B24" s="11" t="s">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="C24" s="11" t="s">
         <v>30</v>
@@ -2728,53 +2879,55 @@
         <v>16.1</v>
       </c>
       <c r="F24" s="11" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="G24" s="9" t="s">
-        <v>76</v>
+        <v>79</v>
       </c>
       <c r="H24" s="11" t="s">
         <v>23</v>
       </c>
-      <c r="J24" s="13"/>
-      <c r="K24" s="13"/>
-      <c r="L24" s="13"/>
+      <c r="I24" s="21"/>
+      <c r="J24" s="22"/>
+      <c r="K24" s="22"/>
+      <c r="L24" s="23"/>
     </row>
     <row r="25" ht="90" spans="1:12">
       <c r="A25" s="9">
         <v>21</v>
       </c>
       <c r="B25" s="11" t="s">
-        <v>94</v>
+        <v>97</v>
       </c>
       <c r="C25" s="10" t="s">
         <v>9</v>
       </c>
       <c r="D25" s="10" t="s">
-        <v>95</v>
+        <v>98</v>
       </c>
       <c r="E25" s="12">
         <v>7.4</v>
       </c>
       <c r="F25" s="11" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="G25" s="9" t="s">
-        <v>76</v>
+        <v>79</v>
       </c>
       <c r="H25" s="11" t="s">
         <v>34</v>
       </c>
-      <c r="J25" s="13"/>
-      <c r="K25" s="13"/>
-      <c r="L25" s="13"/>
+      <c r="I25" s="21"/>
+      <c r="J25" s="22"/>
+      <c r="K25" s="22"/>
+      <c r="L25" s="23"/>
     </row>
     <row r="26" ht="72" spans="1:12">
       <c r="A26" s="9">
         <v>22</v>
       </c>
       <c r="B26" s="11" t="s">
-        <v>96</v>
+        <v>99</v>
       </c>
       <c r="C26" s="10" t="s">
         <v>9</v>
@@ -2786,24 +2939,25 @@
         <v>7.5</v>
       </c>
       <c r="F26" s="11" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="G26" s="9" t="s">
-        <v>76</v>
+        <v>79</v>
       </c>
       <c r="H26" s="11" t="s">
         <v>34</v>
       </c>
-      <c r="J26" s="13"/>
-      <c r="K26" s="13"/>
-      <c r="L26" s="13"/>
+      <c r="I26" s="21"/>
+      <c r="J26" s="22"/>
+      <c r="K26" s="22"/>
+      <c r="L26" s="23"/>
     </row>
     <row r="27" ht="72" spans="1:12">
       <c r="A27" s="9">
         <v>23</v>
       </c>
       <c r="B27" s="11" t="s">
-        <v>97</v>
+        <v>100</v>
       </c>
       <c r="C27" s="10" t="s">
         <v>9</v>
@@ -2815,24 +2969,25 @@
         <v>7.5</v>
       </c>
       <c r="F27" s="11" t="s">
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="G27" s="9" t="s">
-        <v>76</v>
+        <v>79</v>
       </c>
       <c r="H27" s="11" t="s">
         <v>34</v>
       </c>
-      <c r="J27" s="13"/>
-      <c r="K27" s="13"/>
-      <c r="L27" s="13"/>
+      <c r="I27" s="21"/>
+      <c r="J27" s="22"/>
+      <c r="K27" s="22"/>
+      <c r="L27" s="23"/>
     </row>
     <row r="28" ht="72" spans="1:12">
       <c r="A28" s="9">
         <v>24</v>
       </c>
       <c r="B28" s="11" t="s">
-        <v>98</v>
+        <v>101</v>
       </c>
       <c r="C28" s="10" t="s">
         <v>9</v>
@@ -2844,24 +2999,25 @@
         <v>7.5</v>
       </c>
       <c r="F28" s="11" t="s">
-        <v>84</v>
+        <v>87</v>
       </c>
       <c r="G28" s="9" t="s">
-        <v>76</v>
+        <v>79</v>
       </c>
       <c r="H28" s="11" t="s">
         <v>34</v>
       </c>
-      <c r="J28" s="13"/>
-      <c r="K28" s="13"/>
-      <c r="L28" s="13"/>
+      <c r="I28" s="21"/>
+      <c r="J28" s="22"/>
+      <c r="K28" s="22"/>
+      <c r="L28" s="23"/>
     </row>
     <row r="29" ht="72" spans="1:12">
       <c r="A29" s="9">
         <v>25</v>
       </c>
       <c r="B29" s="11" t="s">
-        <v>99</v>
+        <v>102</v>
       </c>
       <c r="C29" s="10" t="s">
         <v>9</v>
@@ -2873,139 +3029,271 @@
         <v>7.5</v>
       </c>
       <c r="F29" s="11" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="G29" s="9" t="s">
-        <v>76</v>
+        <v>79</v>
       </c>
       <c r="H29" s="11" t="s">
         <v>34</v>
       </c>
-      <c r="J29" s="13"/>
-      <c r="K29" s="13"/>
-      <c r="L29" s="13"/>
+      <c r="I29" s="21"/>
+      <c r="J29" s="22"/>
+      <c r="K29" s="22"/>
+      <c r="L29" s="23"/>
     </row>
     <row r="30" ht="72" spans="1:12">
       <c r="A30" s="9">
         <v>26</v>
       </c>
       <c r="B30" s="11" t="s">
-        <v>100</v>
+        <v>103</v>
       </c>
       <c r="C30" s="10" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="D30" s="10" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="E30" s="12">
-        <v>19.9</v>
+        <v>7.5</v>
       </c>
       <c r="F30" s="11" t="s">
-        <v>62</v>
+        <v>72</v>
       </c>
       <c r="G30" s="9" t="s">
-        <v>63</v>
+        <v>79</v>
       </c>
       <c r="H30" s="11" t="s">
-        <v>37</v>
-      </c>
-      <c r="J30" s="13"/>
-      <c r="K30" s="13"/>
-      <c r="L30" s="13"/>
-    </row>
-    <row r="31" ht="54" spans="1:12">
+        <v>34</v>
+      </c>
+      <c r="I30" s="21"/>
+      <c r="J30" s="22"/>
+      <c r="K30" s="22"/>
+      <c r="L30" s="23"/>
+    </row>
+    <row r="31" ht="90" spans="1:12">
       <c r="A31" s="9">
         <v>27</v>
       </c>
       <c r="B31" s="11" t="s">
-        <v>101</v>
+        <v>104</v>
       </c>
       <c r="C31" s="10" t="s">
-        <v>12</v>
+        <v>27</v>
       </c>
       <c r="D31" s="10" t="s">
-        <v>39</v>
+        <v>28</v>
       </c>
       <c r="E31" s="12">
-        <v>19.9</v>
+        <v>23.2</v>
       </c>
       <c r="F31" s="11" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="G31" s="9" t="s">
-        <v>63</v>
+        <v>79</v>
       </c>
       <c r="H31" s="11" t="s">
-        <v>37</v>
-      </c>
-      <c r="J31" s="13"/>
-      <c r="K31" s="13"/>
-      <c r="L31" s="13"/>
-    </row>
-    <row r="32" ht="54" spans="1:12">
+        <v>23</v>
+      </c>
+      <c r="I31" s="21"/>
+      <c r="J31" s="22"/>
+      <c r="K31" s="22"/>
+      <c r="L31" s="23"/>
+    </row>
+    <row r="32" ht="72" spans="1:12">
       <c r="A32" s="9">
         <v>28</v>
       </c>
       <c r="B32" s="11" t="s">
-        <v>102</v>
+        <v>105</v>
       </c>
       <c r="C32" s="10" t="s">
         <v>12</v>
       </c>
       <c r="D32" s="10" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="E32" s="12">
-        <v>19.1</v>
+        <v>19.9</v>
       </c>
       <c r="F32" s="11" t="s">
-        <v>69</v>
+        <v>65</v>
       </c>
       <c r="G32" s="9" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="H32" s="11" t="s">
         <v>37</v>
       </c>
-      <c r="J32" s="13"/>
-      <c r="K32" s="13"/>
-      <c r="L32" s="13"/>
+      <c r="I32" s="21"/>
+      <c r="J32" s="22"/>
+      <c r="K32" s="22"/>
+      <c r="L32" s="23"/>
     </row>
     <row r="33" ht="54" spans="1:12">
       <c r="A33" s="9">
         <v>29</v>
       </c>
       <c r="B33" s="11" t="s">
-        <v>103</v>
+        <v>106</v>
       </c>
       <c r="C33" s="10" t="s">
+        <v>12</v>
+      </c>
+      <c r="D33" s="10" t="s">
+        <v>39</v>
+      </c>
+      <c r="E33" s="12">
+        <v>19.9</v>
+      </c>
+      <c r="F33" s="11" t="s">
+        <v>72</v>
+      </c>
+      <c r="G33" s="9" t="s">
+        <v>66</v>
+      </c>
+      <c r="H33" s="11" t="s">
+        <v>37</v>
+      </c>
+      <c r="I33" s="21"/>
+      <c r="J33" s="22"/>
+      <c r="K33" s="22"/>
+      <c r="L33" s="23"/>
+    </row>
+    <row r="34" ht="54" spans="1:12">
+      <c r="A34" s="9">
+        <v>30</v>
+      </c>
+      <c r="B34" s="11" t="s">
+        <v>107</v>
+      </c>
+      <c r="C34" s="10" t="s">
+        <v>12</v>
+      </c>
+      <c r="D34" s="10" t="s">
+        <v>40</v>
+      </c>
+      <c r="E34" s="12">
+        <v>19.1</v>
+      </c>
+      <c r="F34" s="11" t="s">
+        <v>72</v>
+      </c>
+      <c r="G34" s="9" t="s">
+        <v>66</v>
+      </c>
+      <c r="H34" s="11" t="s">
+        <v>37</v>
+      </c>
+      <c r="I34" s="21"/>
+      <c r="J34" s="22"/>
+      <c r="K34" s="22"/>
+      <c r="L34" s="23"/>
+    </row>
+    <row r="35" ht="54" spans="1:12">
+      <c r="A35" s="9">
+        <v>31</v>
+      </c>
+      <c r="B35" s="11" t="s">
+        <v>108</v>
+      </c>
+      <c r="C35" s="10" t="s">
         <v>42</v>
       </c>
-      <c r="D33" s="10" t="s">
+      <c r="D35" s="10" t="s">
         <v>43</v>
       </c>
-      <c r="E33" s="12">
+      <c r="E35" s="12">
         <v>15.1</v>
       </c>
-      <c r="F33" s="11" t="s">
-        <v>69</v>
-      </c>
-      <c r="G33" s="9" t="s">
-        <v>104</v>
-      </c>
-      <c r="H33" s="11" t="s">
+      <c r="F35" s="11" t="s">
+        <v>72</v>
+      </c>
+      <c r="G35" s="9" t="s">
+        <v>109</v>
+      </c>
+      <c r="H35" s="11" t="s">
         <v>41</v>
       </c>
-      <c r="J33" s="13"/>
-      <c r="K33" s="13"/>
-      <c r="L33" s="13"/>
+      <c r="I35" s="21"/>
+      <c r="J35" s="22"/>
+      <c r="K35" s="22"/>
+      <c r="L35" s="23"/>
+    </row>
+    <row r="36" ht="17.4" spans="1:12">
+      <c r="A36" s="13" t="s">
+        <v>110</v>
+      </c>
+      <c r="B36" s="13"/>
+      <c r="C36" s="13"/>
+      <c r="D36" s="13"/>
+      <c r="E36" s="13"/>
+      <c r="F36" s="13"/>
+      <c r="G36" s="13"/>
+      <c r="H36" s="13"/>
+      <c r="I36" s="18"/>
+      <c r="J36" s="19"/>
+      <c r="K36" s="20"/>
+      <c r="L36" s="23"/>
+    </row>
+    <row r="37" ht="36" spans="1:11">
+      <c r="A37" s="9">
+        <v>32</v>
+      </c>
+      <c r="B37" s="11" t="s">
+        <v>111</v>
+      </c>
+      <c r="C37" s="10"/>
+      <c r="D37" s="10"/>
+      <c r="E37" s="12"/>
+      <c r="F37" s="11" t="s">
+        <v>112</v>
+      </c>
+      <c r="G37" s="9" t="s">
+        <v>66</v>
+      </c>
+      <c r="H37" s="11" t="s">
+        <v>7</v>
+      </c>
+      <c r="I37" s="21"/>
+      <c r="J37" s="21"/>
+      <c r="K37" s="21"/>
+    </row>
+    <row r="38" ht="54" spans="1:11">
+      <c r="A38" s="9">
+        <v>33</v>
+      </c>
+      <c r="B38" s="11" t="s">
+        <v>113</v>
+      </c>
+      <c r="C38" s="10"/>
+      <c r="D38" s="10"/>
+      <c r="E38" s="12"/>
+      <c r="F38" s="11" t="s">
+        <v>112</v>
+      </c>
+      <c r="G38" s="9" t="s">
+        <v>66</v>
+      </c>
+      <c r="H38" s="11" t="s">
+        <v>7</v>
+      </c>
+      <c r="I38" s="21"/>
+      <c r="J38" s="21"/>
+      <c r="K38" s="21"/>
     </row>
   </sheetData>
-  <mergeCells count="3">
-    <mergeCell ref="A1:G1"/>
+  <mergeCells count="8">
+    <mergeCell ref="A1:H1"/>
+    <mergeCell ref="I1:K1"/>
     <mergeCell ref="A3:H3"/>
+    <mergeCell ref="I3:K3"/>
     <mergeCell ref="A15:H15"/>
+    <mergeCell ref="I15:K15"/>
+    <mergeCell ref="A36:H36"/>
+    <mergeCell ref="I36:K36"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter/>

</xml_diff>

<commit_message>
docs : complete result
</commit_message>
<xml_diff>
--- a/sprint_1/1_business_analysis/deliverables/AC.xlsx
+++ b/sprint_1/1_business_analysis/deliverables/AC.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="23040" windowHeight="9707" activeTab="1"/>
+    <workbookView windowWidth="20490" windowHeight="7620" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="364" uniqueCount="175">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="384" uniqueCount="190">
   <si>
     <t>STT</t>
   </si>
@@ -512,12 +512,22 @@
     <t>Tỷ trọng nguồn điện (%) = (Sản lượng điện của từng nguồn / Tổng sản lượng điện toàn hệ thống) / 100.</t>
   </si>
   <si>
+    <t xml:space="preserve"> Công tơ điện tử 2 chiều gồm : 
+- điện đã mua
+ - điện đã tiêu thụ 
+- điện đã tạo ra </t>
+  </si>
+  <si>
     <t xml:space="preserve">Lượng điện tiêu thụ tại [khu vực] </t>
   </si>
   <si>
     <t>Lượng điện tiêu thụ = Tổng kWh tiêu thụ của toàn bộ công tơ tại khu vực trong khoảng thời gian truy vấn.</t>
   </si>
   <si>
+    <t xml:space="preserve">Công tơ điện tử chứa :
+ - điện đã tiêu thụ  trong một khoảng thời gian </t>
+  </si>
+  <si>
     <t>Số liệu/xu hướng sử dụng điện tại [khu vực] trong [số] [ngày/tuần/tháng/năm] qua</t>
   </si>
   <si>
@@ -536,36 +546,56 @@
     <t>Dung lượng lưu trữ của lưới điện hoặc hệ pin lưu trữ / Tổng điện năng tiêu thụ toàn thành phố / 100.</t>
   </si>
   <si>
+    <t xml:space="preserve">Trạm biến áp , Công tơ điện tử chứa :
+ - điện đã tiêu thụ  trong một khoảng thời gian </t>
+  </si>
+  <si>
     <t>Danh sách các nguồn cấp điện bị quá tải</t>
   </si>
   <si>
     <t>Các trạm/nguồn có tải sử dụng vượt ngưỡng cấu hình (ví dụ &gt;80% hoặc &gt;100% công suất thiết kế). Công thức tải (%) = (Công suất hiện tại / Công suất thiết kế) / 100.</t>
   </si>
   <si>
+    <t xml:space="preserve">Trạm biến áp , Công tơ điện tử chứa :
+ - điện đã tiêu thụ  trong một khoảng thời gian và công suất tối đa có thể đáp ứng </t>
+  </si>
+  <si>
     <t>Danh sách các hệ thống cấp nước bị hỏng</t>
   </si>
   <si>
     <t>Lọc các thiết bị/cảm biến/trạm cấp nước có trạng thái lỗi, mất kết nối hoặc không hoạt động.</t>
   </si>
   <si>
+    <t>Các thiết bị cảm biến gửi tín hiệu cập nhật theo ngày</t>
+  </si>
+  <si>
     <t>Số lượng đèn tín hiệu giao thông thông minh hiện tại, lọc theo trạng thái (hoạt động bình thường/hư hỏng)</t>
   </si>
   <si>
     <t>Số đèn thông minh  có trạng thái được hỏi / Tổng số đèn tín hiệu / 100.</t>
   </si>
   <si>
+    <t xml:space="preserve">Tín hiệu từ đèn giao thông và camera gần đó </t>
+  </si>
+  <si>
     <t>Danh sách các đèn báo hiệu giao thông thông minh gặp vấn đề, bị hỏng.</t>
   </si>
   <si>
     <t>Lọc các đèn có trạng thái fault/offline/bảo trì trong hệ thống ITS.</t>
   </si>
   <si>
+    <t xml:space="preserve">Tín hiệu từ đèn giao thông và  người bảo trì </t>
+  </si>
+  <si>
     <t>Các tuyến đường đang ùn tắc hiện tại</t>
   </si>
   <si>
     <t>Xác định tuyến đường hoặc khu vực  có tốc độ trung bình thấp hơn ngưỡng quy định hoặc mật độ phương tiện vượt ngưỡng. Ví dụ: ùn tắc khi tốc độ &lt;20 km/h.</t>
   </si>
   <si>
+    <t xml:space="preserve">Thông tin từ gg map , camera </t>
+  </si>
+  <si>
     <t>Danh sách các camera đang gặp vấn đề, bị hỏng, không hoạt động</t>
   </si>
   <si>
@@ -575,6 +605,9 @@
     <t>Lọc camera có trạng thái offline, mất tín hiệu hoặc lỗi phần cứng/phần mềm.</t>
   </si>
   <si>
+    <t xml:space="preserve">Thông tin dữ liệu từ camera nếu bị ngắt sẽ báo tới quản lí </t>
+  </si>
+  <si>
     <t>PHẦN 2: CÂU HỎI BỔ SUNG THÊM KHÔNG MAPPING VỚI ISO 37122 INDICATOR</t>
   </si>
   <si>
@@ -587,6 +620,9 @@
     <t>Lọc thiết bị access control có trạng thái offline/lỗi/bảo trì theo khu vực.</t>
   </si>
   <si>
+    <t xml:space="preserve"> Thông tin trạng thái các thiết bị từ hạ tầng </t>
+  </si>
+  <si>
     <t>Danh sách các thang máy đang trong trạng thái không hoạt động/hư hỏng/bảo trì</t>
   </si>
   <si>
@@ -605,18 +641,28 @@
     <t>Tổng hợp kWh tiêu thụ theo khu vực và sắp xếp giảm dần</t>
   </si>
   <si>
+    <t xml:space="preserve"> Công tơ điện tử chứa :
+ - điện đã tiêu thụ  trong một khoảng thời gian </t>
+  </si>
+  <si>
     <t>Danh sách các khu vực tiêu thụ nhiều  nước sinh hoạt  nhất</t>
   </si>
   <si>
     <t>Tổng hợp m3 nước tiêu thụ theo khu vực và sắp xếp giảm dần.</t>
   </si>
   <si>
+    <t xml:space="preserve">Công tơ nước chưa : lượng nước đã sử dụng </t>
+  </si>
+  <si>
     <t>Danh sách các khu vực đang có đường thi công , sửa chữa giao thông</t>
   </si>
   <si>
     <t>Lọc các tuyến đường có trạng thái công trình đang hoạt động trong hệ thống quản lý hạ tầng</t>
   </si>
   <si>
+    <t xml:space="preserve"> Thông tin từ người  thi công báo tới ban quản lí </t>
+  </si>
+  <si>
     <t>Danh sách các khu vực đang đang thi công cơ sở hạ tầng (nhà ở ,  bến xe , ... )</t>
   </si>
   <si>
@@ -629,10 +675,16 @@
     <t>Lọc cây xanh có trạng thái hư hại/gãy đổ/sâu bệnh từ hệ thống quản lý cây xanh hoặc phản ánh hiện trường.</t>
   </si>
   <si>
+    <t xml:space="preserve">Thông tin từ quản lí sinh thái báo tới ban quản lí </t>
+  </si>
+  <si>
     <t>Chi phí sửa chữa thiết bị , hạ tầng  của [khu vực] là bao nhiêu tại [thời gian] ?</t>
   </si>
   <si>
     <t>Tổng chi phí vật tư + nhân công + vận hành phát sinh trong khoảng thời gian và khu vực yêu cầu.</t>
+  </si>
+  <si>
+    <t>Hệ thống tổng hợp tài chính gửi lên và đã lưu vào cơ sở dữ liệu</t>
   </si>
 </sst>
 </file>
@@ -2029,18 +2081,18 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:H24"/>
-  <sheetFormatPr defaultColWidth="8.88888888888889" defaultRowHeight="14.4" outlineLevelCol="7"/>
+  <sheetFormatPr defaultColWidth="8.88571428571429" defaultRowHeight="15" outlineLevelCol="7"/>
   <cols>
-    <col min="2" max="2" width="14.1111111111111" customWidth="1"/>
-    <col min="3" max="3" width="28.8888888888889" customWidth="1"/>
-    <col min="4" max="4" width="24.6388888888889" customWidth="1"/>
-    <col min="5" max="5" width="47.4722222222222" customWidth="1"/>
-    <col min="6" max="6" width="19.3888888888889" style="1" customWidth="1"/>
-    <col min="7" max="7" width="12.7314814814815" customWidth="1"/>
-    <col min="8" max="8" width="37.5740740740741" customWidth="1"/>
+    <col min="2" max="2" width="14.1142857142857" customWidth="1"/>
+    <col min="3" max="3" width="28.8857142857143" customWidth="1"/>
+    <col min="4" max="4" width="24.6380952380952" customWidth="1"/>
+    <col min="5" max="5" width="47.4761904761905" customWidth="1"/>
+    <col min="6" max="6" width="19.3904761904762" style="1" customWidth="1"/>
+    <col min="7" max="7" width="12.7333333333333" customWidth="1"/>
+    <col min="8" max="8" width="37.5714285714286" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="17.4" spans="1:8">
+    <row r="1" ht="18.75" spans="1:8">
       <c r="A1" s="28" t="s">
         <v>0</v>
       </c>
@@ -2064,7 +2116,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="2" ht="36" spans="1:8">
+    <row r="2" ht="37.5" spans="1:8">
       <c r="A2" s="10">
         <v>1</v>
       </c>
@@ -2086,7 +2138,7 @@
       <c r="G2" s="30"/>
       <c r="H2" s="30"/>
     </row>
-    <row r="3" ht="36" spans="1:8">
+    <row r="3" ht="37.5" spans="1:8">
       <c r="A3" s="10"/>
       <c r="B3" s="11"/>
       <c r="C3" s="11" t="s">
@@ -2104,7 +2156,7 @@
       <c r="G3" s="30"/>
       <c r="H3" s="30"/>
     </row>
-    <row r="4" ht="36" spans="1:8">
+    <row r="4" ht="37.5" spans="1:8">
       <c r="A4" s="10"/>
       <c r="B4" s="11"/>
       <c r="C4" s="11" t="s">
@@ -2122,7 +2174,7 @@
       <c r="G4" s="30"/>
       <c r="H4" s="30"/>
     </row>
-    <row r="5" ht="36" spans="1:8">
+    <row r="5" ht="37.5" spans="1:8">
       <c r="A5" s="10"/>
       <c r="B5" s="11"/>
       <c r="C5" s="11"/>
@@ -2138,7 +2190,7 @@
       <c r="G5" s="30"/>
       <c r="H5" s="30"/>
     </row>
-    <row r="6" ht="36" spans="1:8">
+    <row r="6" ht="37.5" spans="1:8">
       <c r="A6" s="10"/>
       <c r="B6" s="11"/>
       <c r="C6" s="11"/>
@@ -2154,7 +2206,7 @@
       <c r="G6" s="30"/>
       <c r="H6" s="30"/>
     </row>
-    <row r="7" ht="36" spans="1:8">
+    <row r="7" ht="37.5" spans="1:8">
       <c r="A7" s="10"/>
       <c r="B7" s="11"/>
       <c r="C7" s="11" t="s">
@@ -2172,7 +2224,7 @@
       <c r="G7" s="30"/>
       <c r="H7" s="30"/>
     </row>
-    <row r="8" ht="36" spans="1:8">
+    <row r="8" ht="37.5" spans="1:8">
       <c r="A8" s="10"/>
       <c r="B8" s="11"/>
       <c r="C8" s="11"/>
@@ -2188,7 +2240,7 @@
       <c r="G8" s="30"/>
       <c r="H8" s="30"/>
     </row>
-    <row r="9" ht="54" spans="1:8">
+    <row r="9" ht="56.25" spans="1:8">
       <c r="A9" s="10">
         <v>2</v>
       </c>
@@ -2210,7 +2262,7 @@
       <c r="G9" s="30"/>
       <c r="H9" s="30"/>
     </row>
-    <row r="10" ht="54" spans="1:8">
+    <row r="10" ht="56.25" spans="1:8">
       <c r="A10" s="10"/>
       <c r="B10" s="11"/>
       <c r="C10" s="11" t="s">
@@ -2228,7 +2280,7 @@
       <c r="G10" s="30"/>
       <c r="H10" s="30"/>
     </row>
-    <row r="11" ht="72" spans="1:8">
+    <row r="11" ht="75" spans="1:8">
       <c r="A11" s="10"/>
       <c r="B11" s="11"/>
       <c r="C11" s="11" t="s">
@@ -2246,7 +2298,7 @@
       <c r="G11" s="30"/>
       <c r="H11" s="30"/>
     </row>
-    <row r="12" ht="36" spans="1:8">
+    <row r="12" ht="37.5" spans="1:8">
       <c r="A12" s="10"/>
       <c r="B12" s="11"/>
       <c r="C12" s="11"/>
@@ -2262,7 +2314,7 @@
       <c r="G12" s="30"/>
       <c r="H12" s="30"/>
     </row>
-    <row r="13" ht="36" spans="1:8">
+    <row r="13" ht="37.5" spans="1:8">
       <c r="A13" s="10"/>
       <c r="B13" s="11"/>
       <c r="C13" s="11"/>
@@ -2278,7 +2330,7 @@
       <c r="G13" s="30"/>
       <c r="H13" s="30"/>
     </row>
-    <row r="14" ht="54" spans="1:8">
+    <row r="14" ht="56.25" spans="1:8">
       <c r="A14" s="31">
         <v>3</v>
       </c>
@@ -2298,7 +2350,7 @@
       <c r="G14" s="30"/>
       <c r="H14" s="30"/>
     </row>
-    <row r="15" ht="36" spans="1:8">
+    <row r="15" ht="37.5" spans="1:8">
       <c r="A15" s="32"/>
       <c r="B15" s="11"/>
       <c r="C15" s="11"/>
@@ -2314,7 +2366,7 @@
       <c r="G15" s="30"/>
       <c r="H15" s="30"/>
     </row>
-    <row r="16" ht="36" spans="1:8">
+    <row r="16" ht="37.5" spans="1:8">
       <c r="A16" s="31">
         <v>4</v>
       </c>
@@ -2334,7 +2386,7 @@
       <c r="G16" s="30"/>
       <c r="H16" s="30"/>
     </row>
-    <row r="17" ht="36" spans="1:8">
+    <row r="17" ht="37.5" spans="1:8">
       <c r="A17" s="33"/>
       <c r="B17" s="11"/>
       <c r="C17" s="11"/>
@@ -2350,7 +2402,7 @@
       <c r="G17" s="30"/>
       <c r="H17" s="30"/>
     </row>
-    <row r="18" ht="36" spans="1:8">
+    <row r="18" ht="37.5" spans="1:8">
       <c r="A18" s="32"/>
       <c r="B18" s="11"/>
       <c r="C18" s="11"/>
@@ -2366,7 +2418,7 @@
       <c r="G18" s="30"/>
       <c r="H18" s="30"/>
     </row>
-    <row r="19" ht="36" spans="1:8">
+    <row r="19" ht="37.5" spans="1:8">
       <c r="A19" s="10">
         <v>5</v>
       </c>
@@ -2386,7 +2438,7 @@
       <c r="G19" s="30"/>
       <c r="H19" s="30"/>
     </row>
-    <row r="20" ht="18" spans="1:8">
+    <row r="20" ht="18.75" spans="1:8">
       <c r="A20" s="10">
         <v>6</v>
       </c>
@@ -2404,7 +2456,7 @@
       <c r="G20" s="30"/>
       <c r="H20" s="30"/>
     </row>
-    <row r="21" ht="18" spans="1:8">
+    <row r="21" ht="18.75" spans="1:8">
       <c r="A21" s="10"/>
       <c r="B21" s="11"/>
       <c r="C21" s="11" t="s">
@@ -2418,7 +2470,7 @@
       <c r="G21" s="30"/>
       <c r="H21" s="30"/>
     </row>
-    <row r="22" ht="18" spans="1:8">
+    <row r="22" ht="18.75" spans="1:8">
       <c r="A22" s="10"/>
       <c r="B22" s="11"/>
       <c r="C22" s="11" t="s">
@@ -2432,7 +2484,7 @@
       <c r="G22" s="30"/>
       <c r="H22" s="30"/>
     </row>
-    <row r="23" ht="18" spans="1:8">
+    <row r="23" ht="18.75" spans="1:8">
       <c r="A23" s="10"/>
       <c r="B23" s="11"/>
       <c r="C23" s="11"/>
@@ -2444,7 +2496,7 @@
       <c r="G23" s="30"/>
       <c r="H23" s="30"/>
     </row>
-    <row r="24" ht="36" spans="1:8">
+    <row r="24" ht="37.5" spans="1:8">
       <c r="A24" s="10"/>
       <c r="B24" s="11"/>
       <c r="C24" s="11" t="s">
@@ -2486,22 +2538,22 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:L45"/>
-  <sheetFormatPr defaultColWidth="8.88888888888889" defaultRowHeight="14.4"/>
+  <sheetFormatPr defaultColWidth="8.88571428571429" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="7.31481481481481" customWidth="1"/>
-    <col min="2" max="2" width="36.4444444444444" customWidth="1"/>
-    <col min="3" max="3" width="25.4907407407407" customWidth="1"/>
-    <col min="4" max="4" width="26.0185185185185" customWidth="1"/>
-    <col min="5" max="5" width="19.7037037037037" style="1" customWidth="1"/>
+    <col min="1" max="1" width="7.31428571428571" customWidth="1"/>
+    <col min="2" max="2" width="36.447619047619" customWidth="1"/>
+    <col min="3" max="3" width="25.4952380952381" customWidth="1"/>
+    <col min="4" max="4" width="26.0190476190476" customWidth="1"/>
+    <col min="5" max="5" width="19.7047619047619" style="1" customWidth="1"/>
     <col min="6" max="6" width="29.3333333333333" customWidth="1"/>
-    <col min="7" max="7" width="11.1018518518519" style="1" customWidth="1"/>
-    <col min="8" max="8" width="28.3981481481481" customWidth="1"/>
-    <col min="9" max="9" width="36.1944444444444" style="2" customWidth="1"/>
-    <col min="10" max="10" width="39.2037037037037" style="2" customWidth="1"/>
-    <col min="11" max="11" width="21.8981481481481" style="2" customWidth="1"/>
+    <col min="7" max="7" width="11.1047619047619" style="1" customWidth="1"/>
+    <col min="8" max="8" width="28.4" customWidth="1"/>
+    <col min="9" max="9" width="36.1904761904762" style="2" customWidth="1"/>
+    <col min="10" max="10" width="39.2" style="2" customWidth="1"/>
+    <col min="11" max="11" width="21.8952380952381" style="2" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="17.4" spans="1:11">
+    <row r="1" ht="18.75" spans="1:11">
       <c r="A1" s="3" t="s">
         <v>54</v>
       </c>
@@ -2518,7 +2570,7 @@
       <c r="J1" s="16"/>
       <c r="K1" s="17"/>
     </row>
-    <row r="2" ht="17.4" spans="1:11">
+    <row r="2" ht="37.5" spans="1:11">
       <c r="A2" s="6" t="s">
         <v>0</v>
       </c>
@@ -2553,7 +2605,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="3" ht="18" spans="1:11">
+    <row r="3" ht="18.75" spans="1:11">
       <c r="A3" s="7" t="s">
         <v>63</v>
       </c>
@@ -2568,7 +2620,7 @@
       <c r="J3" s="20"/>
       <c r="K3" s="21"/>
     </row>
-    <row r="4" ht="108" spans="1:11">
+    <row r="4" ht="112.5" spans="1:11">
       <c r="A4" s="10">
         <v>1</v>
       </c>
@@ -2601,7 +2653,7 @@
       </c>
       <c r="K4" s="12"/>
     </row>
-    <row r="5" ht="234" spans="1:11">
+    <row r="5" ht="243.75" spans="1:11">
       <c r="A5" s="10">
         <v>2</v>
       </c>
@@ -2634,7 +2686,7 @@
       </c>
       <c r="K5" s="12"/>
     </row>
-    <row r="6" ht="90" spans="1:11">
+    <row r="6" ht="93.75" spans="1:11">
       <c r="A6" s="10">
         <v>3</v>
       </c>
@@ -2667,7 +2719,7 @@
       </c>
       <c r="K6" s="12"/>
     </row>
-    <row r="7" ht="108" spans="1:11">
+    <row r="7" ht="112.5" spans="1:11">
       <c r="A7" s="10">
         <v>4</v>
       </c>
@@ -2700,7 +2752,7 @@
       </c>
       <c r="K7" s="12"/>
     </row>
-    <row r="8" ht="72" spans="1:11">
+    <row r="8" ht="75" spans="1:11">
       <c r="A8" s="10">
         <v>5</v>
       </c>
@@ -2733,7 +2785,7 @@
       </c>
       <c r="K8" s="12"/>
     </row>
-    <row r="9" ht="108" spans="1:11">
+    <row r="9" ht="112.5" spans="1:11">
       <c r="A9" s="10">
         <v>6</v>
       </c>
@@ -2766,7 +2818,7 @@
       </c>
       <c r="K9" s="12"/>
     </row>
-    <row r="10" ht="108" spans="1:11">
+    <row r="10" ht="112.5" spans="1:11">
       <c r="A10" s="10">
         <v>7</v>
       </c>
@@ -2799,7 +2851,7 @@
       </c>
       <c r="K10" s="12"/>
     </row>
-    <row r="11" ht="108" spans="1:11">
+    <row r="11" ht="112.5" spans="1:11">
       <c r="A11" s="10">
         <v>8</v>
       </c>
@@ -2832,7 +2884,7 @@
       </c>
       <c r="K11" s="12"/>
     </row>
-    <row r="12" ht="90" spans="1:11">
+    <row r="12" ht="93.75" spans="1:11">
       <c r="A12" s="10">
         <v>9</v>
       </c>
@@ -2865,7 +2917,7 @@
       </c>
       <c r="K12" s="12"/>
     </row>
-    <row r="13" ht="108" spans="1:11">
+    <row r="13" ht="112.5" spans="1:11">
       <c r="A13" s="10">
         <v>10</v>
       </c>
@@ -2898,7 +2950,7 @@
       </c>
       <c r="K13" s="12"/>
     </row>
-    <row r="14" ht="108" spans="1:11">
+    <row r="14" ht="112.5" spans="1:11">
       <c r="A14" s="10">
         <v>11</v>
       </c>
@@ -2931,7 +2983,7 @@
       </c>
       <c r="K14" s="12"/>
     </row>
-    <row r="15" ht="18" spans="1:11">
+    <row r="15" ht="18.75" spans="1:11">
       <c r="A15" s="14" t="s">
         <v>103</v>
       </c>
@@ -2946,7 +2998,7 @@
       <c r="J15" s="23"/>
       <c r="K15" s="24"/>
     </row>
-    <row r="16" ht="108" spans="1:12">
+    <row r="16" ht="112.5" spans="1:12">
       <c r="A16" s="10">
         <v>12</v>
       </c>
@@ -2980,7 +3032,7 @@
       <c r="K16" s="12"/>
       <c r="L16" s="2"/>
     </row>
-    <row r="17" ht="72" spans="1:12">
+    <row r="17" ht="75" spans="1:12">
       <c r="A17" s="10">
         <v>13</v>
       </c>
@@ -3014,7 +3066,7 @@
       <c r="K17" s="12"/>
       <c r="L17" s="2"/>
     </row>
-    <row r="18" ht="72" spans="1:12">
+    <row r="18" ht="75" spans="1:12">
       <c r="A18" s="10">
         <v>14</v>
       </c>
@@ -3048,7 +3100,7 @@
       <c r="K18" s="12"/>
       <c r="L18" s="2"/>
     </row>
-    <row r="19" ht="108" spans="1:12">
+    <row r="19" ht="112.5" spans="1:12">
       <c r="A19" s="10">
         <v>15</v>
       </c>
@@ -3082,7 +3134,7 @@
       <c r="K19" s="12"/>
       <c r="L19" s="2"/>
     </row>
-    <row r="20" ht="216" spans="1:12">
+    <row r="20" ht="225" spans="1:12">
       <c r="A20" s="10">
         <v>16</v>
       </c>
@@ -3116,7 +3168,7 @@
       <c r="K20" s="12"/>
       <c r="L20" s="2"/>
     </row>
-    <row r="21" ht="108" spans="1:12">
+    <row r="21" ht="112.5" spans="1:12">
       <c r="A21" s="10">
         <v>17</v>
       </c>
@@ -3150,7 +3202,7 @@
       <c r="K21" s="12"/>
       <c r="L21" s="2"/>
     </row>
-    <row r="22" ht="108" spans="1:12">
+    <row r="22" ht="112.5" spans="1:12">
       <c r="A22" s="10">
         <v>18</v>
       </c>
@@ -3184,7 +3236,7 @@
       <c r="K22" s="12"/>
       <c r="L22" s="2"/>
     </row>
-    <row r="23" ht="180" spans="1:12">
+    <row r="23" ht="187.5" spans="1:12">
       <c r="A23" s="10">
         <v>19</v>
       </c>
@@ -3216,7 +3268,7 @@
       <c r="K23" s="12"/>
       <c r="L23" s="2"/>
     </row>
-    <row r="24" ht="72" spans="1:12">
+    <row r="24" ht="75" spans="1:12">
       <c r="A24" s="10">
         <v>20</v>
       </c>
@@ -3248,7 +3300,7 @@
       <c r="K24" s="12"/>
       <c r="L24" s="2"/>
     </row>
-    <row r="25" ht="90" spans="1:12">
+    <row r="25" ht="93.75" spans="1:12">
       <c r="A25" s="10">
         <v>21</v>
       </c>
@@ -3276,16 +3328,18 @@
       <c r="I25" s="12" t="s">
         <v>133</v>
       </c>
-      <c r="J25" s="12"/>
+      <c r="J25" s="12" t="s">
+        <v>134</v>
+      </c>
       <c r="K25" s="12"/>
       <c r="L25" s="2"/>
     </row>
-    <row r="26" ht="72" spans="1:12">
+    <row r="26" ht="75" spans="1:12">
       <c r="A26" s="10">
         <v>22</v>
       </c>
       <c r="B26" s="12" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="C26" s="11" t="s">
         <v>9</v>
@@ -3306,18 +3360,20 @@
         <v>34</v>
       </c>
       <c r="I26" s="12" t="s">
-        <v>135</v>
-      </c>
-      <c r="J26" s="12"/>
+        <v>136</v>
+      </c>
+      <c r="J26" s="12" t="s">
+        <v>137</v>
+      </c>
       <c r="K26" s="12"/>
       <c r="L26" s="2"/>
     </row>
-    <row r="27" ht="72" spans="1:12">
+    <row r="27" ht="75" spans="1:12">
       <c r="A27" s="10">
         <v>23</v>
       </c>
       <c r="B27" s="12" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="C27" s="11" t="s">
         <v>9</v>
@@ -3338,18 +3394,20 @@
         <v>34</v>
       </c>
       <c r="I27" s="12" t="s">
+        <v>139</v>
+      </c>
+      <c r="J27" s="12" t="s">
         <v>137</v>
       </c>
-      <c r="J27" s="12"/>
       <c r="K27" s="12"/>
       <c r="L27" s="2"/>
     </row>
-    <row r="28" ht="72" spans="1:12">
+    <row r="28" ht="75" spans="1:12">
       <c r="A28" s="10">
         <v>24</v>
       </c>
       <c r="B28" s="12" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="C28" s="11" t="s">
         <v>9</v>
@@ -3370,18 +3428,20 @@
         <v>34</v>
       </c>
       <c r="I28" s="12" t="s">
-        <v>139</v>
-      </c>
-      <c r="J28" s="12"/>
+        <v>141</v>
+      </c>
+      <c r="J28" s="12" t="s">
+        <v>137</v>
+      </c>
       <c r="K28" s="12"/>
       <c r="L28" s="2"/>
     </row>
-    <row r="29" ht="72" spans="1:12">
+    <row r="29" ht="75" spans="1:12">
       <c r="A29" s="10">
         <v>25</v>
       </c>
       <c r="B29" s="12" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="C29" s="11" t="s">
         <v>9</v>
@@ -3402,18 +3462,20 @@
         <v>34</v>
       </c>
       <c r="I29" s="12" t="s">
-        <v>141</v>
-      </c>
-      <c r="J29" s="12"/>
+        <v>143</v>
+      </c>
+      <c r="J29" s="12" t="s">
+        <v>144</v>
+      </c>
       <c r="K29" s="12"/>
       <c r="L29" s="2"/>
     </row>
-    <row r="30" ht="108" spans="1:12">
+    <row r="30" ht="112.5" spans="1:12">
       <c r="A30" s="10">
         <v>26</v>
       </c>
       <c r="B30" s="12" t="s">
-        <v>142</v>
+        <v>145</v>
       </c>
       <c r="C30" s="11" t="s">
         <v>9</v>
@@ -3434,18 +3496,20 @@
         <v>34</v>
       </c>
       <c r="I30" s="12" t="s">
-        <v>143</v>
-      </c>
-      <c r="J30" s="12"/>
+        <v>146</v>
+      </c>
+      <c r="J30" s="12" t="s">
+        <v>147</v>
+      </c>
       <c r="K30" s="12"/>
       <c r="L30" s="2"/>
     </row>
-    <row r="31" ht="90" spans="1:12">
+    <row r="31" ht="93.75" spans="1:12">
       <c r="A31" s="10">
         <v>27</v>
       </c>
       <c r="B31" s="12" t="s">
-        <v>144</v>
+        <v>148</v>
       </c>
       <c r="C31" s="11" t="s">
         <v>27</v>
@@ -3466,18 +3530,20 @@
         <v>23</v>
       </c>
       <c r="I31" s="12" t="s">
-        <v>145</v>
-      </c>
-      <c r="J31" s="12"/>
+        <v>149</v>
+      </c>
+      <c r="J31" s="12" t="s">
+        <v>150</v>
+      </c>
       <c r="K31" s="12"/>
       <c r="L31" s="2"/>
     </row>
-    <row r="32" ht="72" spans="1:12">
+    <row r="32" ht="75" spans="1:12">
       <c r="A32" s="10">
         <v>28</v>
       </c>
       <c r="B32" s="12" t="s">
-        <v>146</v>
+        <v>151</v>
       </c>
       <c r="C32" s="11" t="s">
         <v>12</v>
@@ -3498,18 +3564,20 @@
         <v>37</v>
       </c>
       <c r="I32" s="12" t="s">
-        <v>147</v>
-      </c>
-      <c r="J32" s="12"/>
+        <v>152</v>
+      </c>
+      <c r="J32" s="12" t="s">
+        <v>153</v>
+      </c>
       <c r="K32" s="12"/>
       <c r="L32" s="2"/>
     </row>
-    <row r="33" ht="54" spans="1:12">
+    <row r="33" ht="56.25" spans="1:12">
       <c r="A33" s="10">
         <v>29</v>
       </c>
       <c r="B33" s="12" t="s">
-        <v>148</v>
+        <v>154</v>
       </c>
       <c r="C33" s="11" t="s">
         <v>12</v>
@@ -3530,18 +3598,20 @@
         <v>37</v>
       </c>
       <c r="I33" s="12" t="s">
-        <v>149</v>
-      </c>
-      <c r="J33" s="12"/>
+        <v>155</v>
+      </c>
+      <c r="J33" s="12" t="s">
+        <v>156</v>
+      </c>
       <c r="K33" s="12"/>
       <c r="L33" s="2"/>
     </row>
-    <row r="34" ht="90" spans="1:12">
+    <row r="34" ht="93.75" spans="1:12">
       <c r="A34" s="10">
         <v>30</v>
       </c>
       <c r="B34" s="12" t="s">
-        <v>150</v>
+        <v>157</v>
       </c>
       <c r="C34" s="11" t="s">
         <v>12</v>
@@ -3562,18 +3632,20 @@
         <v>37</v>
       </c>
       <c r="I34" s="12" t="s">
-        <v>151</v>
-      </c>
-      <c r="J34" s="12"/>
+        <v>158</v>
+      </c>
+      <c r="J34" s="12" t="s">
+        <v>159</v>
+      </c>
       <c r="K34" s="12"/>
       <c r="L34" s="2"/>
     </row>
-    <row r="35" ht="54" spans="1:12">
+    <row r="35" ht="56.25" spans="1:12">
       <c r="A35" s="10">
         <v>31</v>
       </c>
       <c r="B35" s="12" t="s">
-        <v>152</v>
+        <v>160</v>
       </c>
       <c r="C35" s="11" t="s">
         <v>42</v>
@@ -3588,21 +3660,23 @@
         <v>79</v>
       </c>
       <c r="G35" s="10" t="s">
-        <v>153</v>
+        <v>161</v>
       </c>
       <c r="H35" s="12" t="s">
         <v>41</v>
       </c>
       <c r="I35" s="12" t="s">
-        <v>154</v>
-      </c>
-      <c r="J35" s="12"/>
+        <v>162</v>
+      </c>
+      <c r="J35" s="12" t="s">
+        <v>163</v>
+      </c>
       <c r="K35" s="12"/>
       <c r="L35" s="2"/>
     </row>
-    <row r="36" ht="18" spans="1:12">
+    <row r="36" ht="18.75" spans="1:12">
       <c r="A36" s="14" t="s">
-        <v>155</v>
+        <v>164</v>
       </c>
       <c r="B36" s="14"/>
       <c r="C36" s="14"/>
@@ -3616,18 +3690,18 @@
       <c r="K36" s="27"/>
       <c r="L36" s="2"/>
     </row>
-    <row r="37" ht="54" spans="1:11">
+    <row r="37" ht="56.25" spans="1:11">
       <c r="A37" s="10">
         <v>32</v>
       </c>
       <c r="B37" s="12" t="s">
-        <v>156</v>
+        <v>165</v>
       </c>
       <c r="C37" s="11"/>
       <c r="D37" s="11"/>
       <c r="E37" s="13"/>
       <c r="F37" s="12" t="s">
-        <v>157</v>
+        <v>166</v>
       </c>
       <c r="G37" s="10" t="s">
         <v>66</v>
@@ -3636,23 +3710,25 @@
         <v>7</v>
       </c>
       <c r="I37" s="12" t="s">
-        <v>158</v>
-      </c>
-      <c r="J37" s="12"/>
+        <v>167</v>
+      </c>
+      <c r="J37" s="12" t="s">
+        <v>168</v>
+      </c>
       <c r="K37" s="12"/>
     </row>
-    <row r="38" ht="54" spans="1:11">
+    <row r="38" ht="56.25" spans="1:11">
       <c r="A38" s="10">
         <v>33</v>
       </c>
       <c r="B38" s="12" t="s">
-        <v>159</v>
+        <v>169</v>
       </c>
       <c r="C38" s="11"/>
       <c r="D38" s="11"/>
       <c r="E38" s="13"/>
       <c r="F38" s="12" t="s">
-        <v>157</v>
+        <v>166</v>
       </c>
       <c r="G38" s="10" t="s">
         <v>66</v>
@@ -3661,9 +3737,11 @@
         <v>7</v>
       </c>
       <c r="I38" s="12" t="s">
-        <v>160</v>
-      </c>
-      <c r="J38" s="12"/>
+        <v>170</v>
+      </c>
+      <c r="J38" s="12" t="s">
+        <v>168</v>
+      </c>
       <c r="K38" s="12"/>
     </row>
     <row r="39" ht="79" customHeight="1" spans="1:11">
@@ -3671,13 +3749,13 @@
         <v>34</v>
       </c>
       <c r="B39" s="12" t="s">
-        <v>161</v>
+        <v>171</v>
       </c>
       <c r="C39" s="11"/>
       <c r="D39" s="11"/>
       <c r="E39" s="13"/>
       <c r="F39" s="12" t="s">
-        <v>157</v>
+        <v>166</v>
       </c>
       <c r="G39" s="10" t="s">
         <v>66</v>
@@ -3686,23 +3764,25 @@
         <v>7</v>
       </c>
       <c r="I39" s="12" t="s">
-        <v>162</v>
-      </c>
-      <c r="J39" s="12"/>
+        <v>172</v>
+      </c>
+      <c r="J39" s="12" t="s">
+        <v>168</v>
+      </c>
       <c r="K39" s="12"/>
     </row>
-    <row r="40" ht="36" spans="1:11">
+    <row r="40" ht="56.25" spans="1:11">
       <c r="A40" s="10">
         <v>35</v>
       </c>
       <c r="B40" s="12" t="s">
-        <v>163</v>
+        <v>173</v>
       </c>
       <c r="C40" s="11"/>
       <c r="D40" s="11"/>
       <c r="E40" s="13"/>
       <c r="F40" s="12" t="s">
-        <v>157</v>
+        <v>166</v>
       </c>
       <c r="G40" s="10" t="s">
         <v>66</v>
@@ -3711,23 +3791,25 @@
         <v>7</v>
       </c>
       <c r="I40" s="12" t="s">
-        <v>164</v>
-      </c>
-      <c r="J40" s="12"/>
+        <v>174</v>
+      </c>
+      <c r="J40" s="12" t="s">
+        <v>175</v>
+      </c>
       <c r="K40" s="12"/>
     </row>
-    <row r="41" ht="36" spans="1:11">
+    <row r="41" ht="37.5" spans="1:11">
       <c r="A41" s="10">
         <v>36</v>
       </c>
       <c r="B41" s="12" t="s">
-        <v>165</v>
+        <v>176</v>
       </c>
       <c r="C41" s="11"/>
       <c r="D41" s="11"/>
       <c r="E41" s="13"/>
       <c r="F41" s="12" t="s">
-        <v>157</v>
+        <v>166</v>
       </c>
       <c r="G41" s="10" t="s">
         <v>66</v>
@@ -3736,23 +3818,25 @@
         <v>7</v>
       </c>
       <c r="I41" s="12" t="s">
-        <v>166</v>
-      </c>
-      <c r="J41" s="12"/>
+        <v>177</v>
+      </c>
+      <c r="J41" s="12" t="s">
+        <v>178</v>
+      </c>
       <c r="K41" s="12"/>
     </row>
-    <row r="42" ht="54" spans="1:11">
+    <row r="42" ht="56.25" spans="1:11">
       <c r="A42" s="10">
         <v>37</v>
       </c>
       <c r="B42" s="12" t="s">
-        <v>167</v>
+        <v>179</v>
       </c>
       <c r="C42" s="11"/>
       <c r="D42" s="11"/>
       <c r="E42" s="13"/>
       <c r="F42" s="12" t="s">
-        <v>157</v>
+        <v>166</v>
       </c>
       <c r="G42" s="10" t="s">
         <v>66</v>
@@ -3761,23 +3845,25 @@
         <v>7</v>
       </c>
       <c r="I42" s="12" t="s">
-        <v>168</v>
-      </c>
-      <c r="J42" s="12"/>
+        <v>180</v>
+      </c>
+      <c r="J42" s="12" t="s">
+        <v>181</v>
+      </c>
       <c r="K42" s="12"/>
     </row>
-    <row r="43" ht="54" spans="1:11">
+    <row r="43" ht="56.25" spans="1:11">
       <c r="A43" s="10">
         <v>38</v>
       </c>
       <c r="B43" s="12" t="s">
-        <v>169</v>
+        <v>182</v>
       </c>
       <c r="C43" s="11"/>
       <c r="D43" s="11"/>
       <c r="E43" s="13"/>
       <c r="F43" s="12" t="s">
-        <v>157</v>
+        <v>166</v>
       </c>
       <c r="G43" s="10" t="s">
         <v>66</v>
@@ -3786,23 +3872,25 @@
         <v>7</v>
       </c>
       <c r="I43" s="12" t="s">
-        <v>170</v>
-      </c>
-      <c r="J43" s="12"/>
+        <v>183</v>
+      </c>
+      <c r="J43" s="12" t="s">
+        <v>181</v>
+      </c>
       <c r="K43" s="12"/>
     </row>
-    <row r="44" ht="72" spans="1:11">
+    <row r="44" ht="75" spans="1:11">
       <c r="A44" s="10">
         <v>39</v>
       </c>
       <c r="B44" s="12" t="s">
-        <v>171</v>
+        <v>184</v>
       </c>
       <c r="C44" s="11"/>
       <c r="D44" s="11"/>
       <c r="E44" s="13"/>
       <c r="F44" s="12" t="s">
-        <v>157</v>
+        <v>166</v>
       </c>
       <c r="G44" s="10" t="s">
         <v>66</v>
@@ -3811,23 +3899,25 @@
         <v>7</v>
       </c>
       <c r="I44" s="12" t="s">
-        <v>172</v>
-      </c>
-      <c r="J44" s="12"/>
+        <v>185</v>
+      </c>
+      <c r="J44" s="12" t="s">
+        <v>186</v>
+      </c>
       <c r="K44" s="12"/>
     </row>
-    <row r="45" ht="54" spans="1:11">
+    <row r="45" ht="75" spans="1:11">
       <c r="A45" s="10">
         <v>40</v>
       </c>
       <c r="B45" s="12" t="s">
-        <v>173</v>
+        <v>187</v>
       </c>
       <c r="C45" s="11"/>
       <c r="D45" s="11"/>
       <c r="E45" s="13"/>
       <c r="F45" s="12" t="s">
-        <v>157</v>
+        <v>166</v>
       </c>
       <c r="G45" s="10" t="s">
         <v>66</v>
@@ -3836,9 +3926,11 @@
         <v>7</v>
       </c>
       <c r="I45" s="12" t="s">
-        <v>174</v>
-      </c>
-      <c r="J45" s="12"/>
+        <v>188</v>
+      </c>
+      <c r="J45" s="12" t="s">
+        <v>189</v>
+      </c>
       <c r="K45" s="12"/>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
update review sprint 1.1 AC
</commit_message>
<xml_diff>
--- a/sprint_1/1_business_analysis/deliverables/AC.xlsx
+++ b/sprint_1/1_business_analysis/deliverables/AC.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="20490" windowHeight="7620" activeTab="1"/>
+    <workbookView windowWidth="23040" windowHeight="9707" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="384" uniqueCount="190">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="412" uniqueCount="202">
   <si>
     <t>STT</t>
   </si>
@@ -221,6 +221,12 @@
   </si>
   <si>
     <t xml:space="preserve">PHẦN 1: CÂU HỎI CHO CƯ DÂN (RESIDENT) </t>
+  </si>
+  <si>
+    <t>Technical</t>
+  </si>
+  <si>
+    <t>Business</t>
   </si>
   <si>
     <t>Kiếm trạm sạc xe điện gần [vị trí]</t>
@@ -282,6 +288,15 @@
 - Tính khoảng cách</t>
   </si>
   <si>
+    <t>x</t>
+  </si>
+  <si>
+    <t>Xe máy không 100% chính xác, nên narrow down cho xe ô tô)</t>
+  </si>
+  <si>
+    <t>Chỉ có 1 bãi xe</t>
+  </si>
+  <si>
     <t>Bãi xe [tên/vị trí] còn chỗ trống không</t>
   </si>
   <si>
@@ -298,7 +313,7 @@
 - Slot available</t>
   </si>
   <si>
-    <t>Số liệu tiêu thụ điện của hộ gia đình tôi trong [số] tháng qua?</t>
+    <t>Số liệu tiêu thụ điện của [khu vực] trong [số] tháng qua?</t>
   </si>
   <si>
     <t>Trả về số liệu công tơ điện theo từng tháng
@@ -313,7 +328,10 @@
 - Timestamp</t>
   </si>
   <si>
-    <t>Số liệu tiêu thụ nước của hộ gia đình tôi trong [số] tháng qua?</t>
+    <t>Khu vuc tinh theo toa nha</t>
+  </si>
+  <si>
+    <t>Số liệu tiêu thụ nước của [khu vực] trong [số] tháng qua?</t>
   </si>
   <si>
     <t>Trả về số liệu công tơ nước theo từng tháng
@@ -350,6 +368,9 @@
 - Status</t>
   </si>
   <si>
+    <t>Lam rõ thế nào là thiết bị thông minh</t>
+  </si>
+  <si>
     <t xml:space="preserve">Tòa nhà [tên/vị trí] có thiết bị lọc/kiểm tra không khí trong nhà không? </t>
   </si>
   <si>
@@ -459,6 +480,12 @@
 - Loại xe</t>
   </si>
   <si>
+    <t>0- do không có số liệu đăng ký xe của cư dân</t>
+  </si>
+  <si>
+    <t>Kiểm tra độ phủ, đánh giá xem có nhận thêm xe không</t>
+  </si>
+  <si>
     <t>Top [số] bãi xe được sử dụng [ít/nhiều] nhất</t>
   </si>
   <si>
@@ -473,6 +500,9 @@
 - Action log (xe ra, xe vào)</t>
   </si>
   <si>
+    <t>Đánh giá lại metrics đo mức sử dụng cảu parking lot</t>
+  </si>
+  <si>
     <t>Danh sách các thiết bị thông minh lắp đặt trong nhà bị hư hỏng</t>
   </si>
   <si>
@@ -528,6 +558,9 @@
  - điện đã tiêu thụ  trong một khoảng thời gian </t>
   </si>
   <si>
+    <t>tòa nhà</t>
+  </si>
+  <si>
     <t>Số liệu/xu hướng sử dụng điện tại [khu vực] trong [số] [ngày/tuần/tháng/năm] qua</t>
   </si>
   <si>
@@ -643,6 +676,9 @@
   <si>
     <t xml:space="preserve"> Công tơ điện tử chứa :
  - điện đã tiêu thụ  trong một khoảng thời gian </t>
+  </si>
+  <si>
+    <t>trùng</t>
   </si>
   <si>
     <t>Danh sách các khu vực tiêu thụ nhiều  nước sinh hoạt  nhất</t>
@@ -1444,7 +1480,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="34">
+  <cellXfs count="35">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -1453,6 +1489,9 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -2081,434 +2120,434 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
   <dimension ref="A1:H24"/>
-  <sheetFormatPr defaultColWidth="8.88571428571429" defaultRowHeight="15" outlineLevelCol="7"/>
+  <sheetFormatPr defaultColWidth="8.88888888888889" defaultRowHeight="14.4" outlineLevelCol="7"/>
   <cols>
-    <col min="2" max="2" width="14.1142857142857" customWidth="1"/>
-    <col min="3" max="3" width="28.8857142857143" customWidth="1"/>
-    <col min="4" max="4" width="24.6380952380952" customWidth="1"/>
-    <col min="5" max="5" width="47.4761904761905" customWidth="1"/>
-    <col min="6" max="6" width="19.3904761904762" style="1" customWidth="1"/>
-    <col min="7" max="7" width="12.7333333333333" customWidth="1"/>
-    <col min="8" max="8" width="37.5714285714286" customWidth="1"/>
+    <col min="2" max="2" width="14.1111111111111" customWidth="1"/>
+    <col min="3" max="3" width="28.8888888888889" customWidth="1"/>
+    <col min="4" max="4" width="24.6388888888889" customWidth="1"/>
+    <col min="5" max="5" width="47.4722222222222" customWidth="1"/>
+    <col min="6" max="6" width="19.3888888888889" style="1" customWidth="1"/>
+    <col min="7" max="7" width="12.7314814814815" customWidth="1"/>
+    <col min="8" max="8" width="37.5740740740741" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="18.75" spans="1:8">
-      <c r="A1" s="28" t="s">
+    <row r="1" ht="17.4" spans="1:8">
+      <c r="A1" s="29" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="28" t="s">
+      <c r="B1" s="29" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="28"/>
-      <c r="D1" s="28" t="s">
+      <c r="C1" s="29"/>
+      <c r="D1" s="29" t="s">
         <v>2</v>
       </c>
-      <c r="E1" s="28" t="s">
+      <c r="E1" s="29" t="s">
         <v>3</v>
       </c>
-      <c r="F1" s="29" t="s">
+      <c r="F1" s="30" t="s">
         <v>4</v>
       </c>
-      <c r="G1" s="29" t="s">
+      <c r="G1" s="30" t="s">
         <v>5</v>
       </c>
-      <c r="H1" s="29" t="s">
+      <c r="H1" s="30" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="2" ht="37.5" spans="1:8">
-      <c r="A2" s="10">
+    <row r="2" ht="36" spans="1:8">
+      <c r="A2" s="11">
         <v>1</v>
       </c>
-      <c r="B2" s="11" t="s">
+      <c r="B2" s="12" t="s">
         <v>7</v>
       </c>
-      <c r="C2" s="11" t="s">
+      <c r="C2" s="12" t="s">
         <v>8</v>
       </c>
-      <c r="D2" s="11" t="s">
+      <c r="D2" s="12" t="s">
         <v>9</v>
       </c>
-      <c r="E2" s="11" t="s">
+      <c r="E2" s="12" t="s">
         <v>10</v>
       </c>
-      <c r="F2" s="13">
+      <c r="F2" s="14">
         <v>7.1</v>
       </c>
-      <c r="G2" s="30"/>
-      <c r="H2" s="30"/>
-    </row>
-    <row r="3" ht="37.5" spans="1:8">
-      <c r="A3" s="10"/>
-      <c r="B3" s="11"/>
-      <c r="C3" s="11" t="s">
+      <c r="G2" s="31"/>
+      <c r="H2" s="31"/>
+    </row>
+    <row r="3" ht="36" spans="1:8">
+      <c r="A3" s="11"/>
+      <c r="B3" s="12"/>
+      <c r="C3" s="12" t="s">
         <v>11</v>
       </c>
-      <c r="D3" s="11" t="s">
+      <c r="D3" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="E3" s="11" t="s">
+      <c r="E3" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="F3" s="13">
+      <c r="F3" s="14">
         <v>19.8</v>
       </c>
-      <c r="G3" s="30"/>
-      <c r="H3" s="30"/>
-    </row>
-    <row r="4" ht="37.5" spans="1:8">
-      <c r="A4" s="10"/>
-      <c r="B4" s="11"/>
-      <c r="C4" s="11" t="s">
+      <c r="G3" s="31"/>
+      <c r="H3" s="31"/>
+    </row>
+    <row r="4" ht="36" spans="1:8">
+      <c r="A4" s="11"/>
+      <c r="B4" s="12"/>
+      <c r="C4" s="12" t="s">
         <v>14</v>
       </c>
-      <c r="D4" s="12" t="s">
+      <c r="D4" s="13" t="s">
         <v>15</v>
       </c>
-      <c r="E4" s="11" t="s">
+      <c r="E4" s="12" t="s">
         <v>16</v>
       </c>
-      <c r="F4" s="13">
+      <c r="F4" s="14">
         <v>12.1</v>
       </c>
-      <c r="G4" s="30"/>
-      <c r="H4" s="30"/>
-    </row>
-    <row r="5" ht="37.5" spans="1:8">
-      <c r="A5" s="10"/>
-      <c r="B5" s="11"/>
-      <c r="C5" s="11"/>
-      <c r="D5" s="12" t="s">
+      <c r="G4" s="31"/>
+      <c r="H4" s="31"/>
+    </row>
+    <row r="5" ht="36" spans="1:8">
+      <c r="A5" s="11"/>
+      <c r="B5" s="12"/>
+      <c r="C5" s="12"/>
+      <c r="D5" s="13" t="s">
         <v>15</v>
       </c>
-      <c r="E5" s="11" t="s">
+      <c r="E5" s="12" t="s">
         <v>17</v>
       </c>
-      <c r="F5" s="13">
+      <c r="F5" s="14">
         <v>12.2</v>
       </c>
-      <c r="G5" s="30"/>
-      <c r="H5" s="30"/>
-    </row>
-    <row r="6" ht="37.5" spans="1:8">
-      <c r="A6" s="10"/>
-      <c r="B6" s="11"/>
-      <c r="C6" s="11"/>
-      <c r="D6" s="11" t="s">
+      <c r="G5" s="31"/>
+      <c r="H5" s="31"/>
+    </row>
+    <row r="6" ht="36" spans="1:8">
+      <c r="A6" s="11"/>
+      <c r="B6" s="12"/>
+      <c r="C6" s="12"/>
+      <c r="D6" s="12" t="s">
         <v>18</v>
       </c>
-      <c r="E6" s="11" t="s">
+      <c r="E6" s="12" t="s">
         <v>19</v>
       </c>
-      <c r="F6" s="13">
+      <c r="F6" s="14">
         <v>8.3</v>
       </c>
-      <c r="G6" s="30"/>
-      <c r="H6" s="30"/>
-    </row>
-    <row r="7" ht="37.5" spans="1:8">
-      <c r="A7" s="10"/>
-      <c r="B7" s="11"/>
-      <c r="C7" s="11" t="s">
+      <c r="G6" s="31"/>
+      <c r="H6" s="31"/>
+    </row>
+    <row r="7" ht="36" spans="1:8">
+      <c r="A7" s="11"/>
+      <c r="B7" s="12"/>
+      <c r="C7" s="12" t="s">
         <v>20</v>
       </c>
-      <c r="D7" s="11" t="s">
+      <c r="D7" s="12" t="s">
         <v>9</v>
       </c>
-      <c r="E7" s="11" t="s">
+      <c r="E7" s="12" t="s">
         <v>21</v>
       </c>
-      <c r="F7" s="13">
+      <c r="F7" s="14">
         <v>7.6</v>
       </c>
-      <c r="G7" s="30"/>
-      <c r="H7" s="30"/>
-    </row>
-    <row r="8" ht="37.5" spans="1:8">
-      <c r="A8" s="10"/>
-      <c r="B8" s="11"/>
-      <c r="C8" s="11"/>
-      <c r="D8" s="11" t="s">
+      <c r="G7" s="31"/>
+      <c r="H7" s="31"/>
+    </row>
+    <row r="8" ht="36" spans="1:8">
+      <c r="A8" s="11"/>
+      <c r="B8" s="12"/>
+      <c r="C8" s="12"/>
+      <c r="D8" s="12" t="s">
         <v>9</v>
       </c>
-      <c r="E8" s="11" t="s">
+      <c r="E8" s="12" t="s">
         <v>22</v>
       </c>
-      <c r="F8" s="13">
+      <c r="F8" s="14">
         <v>7.7</v>
       </c>
-      <c r="G8" s="30"/>
-      <c r="H8" s="30"/>
-    </row>
-    <row r="9" ht="56.25" spans="1:8">
-      <c r="A9" s="10">
+      <c r="G8" s="31"/>
+      <c r="H8" s="31"/>
+    </row>
+    <row r="9" ht="54" spans="1:8">
+      <c r="A9" s="11">
         <v>2</v>
       </c>
-      <c r="B9" s="11" t="s">
+      <c r="B9" s="12" t="s">
         <v>23</v>
       </c>
-      <c r="C9" s="11" t="s">
+      <c r="C9" s="12" t="s">
         <v>24</v>
       </c>
-      <c r="D9" s="11" t="s">
+      <c r="D9" s="12" t="s">
         <v>18</v>
       </c>
-      <c r="E9" s="11" t="s">
+      <c r="E9" s="12" t="s">
         <v>25</v>
       </c>
-      <c r="F9" s="13">
+      <c r="F9" s="14">
         <v>8.2</v>
       </c>
-      <c r="G9" s="30"/>
-      <c r="H9" s="30"/>
-    </row>
-    <row r="10" ht="56.25" spans="1:8">
-      <c r="A10" s="10"/>
-      <c r="B10" s="11"/>
-      <c r="C10" s="11" t="s">
+      <c r="G9" s="31"/>
+      <c r="H9" s="31"/>
+    </row>
+    <row r="10" ht="54" spans="1:8">
+      <c r="A10" s="11"/>
+      <c r="B10" s="12"/>
+      <c r="C10" s="12" t="s">
         <v>26</v>
       </c>
-      <c r="D10" s="11" t="s">
+      <c r="D10" s="12" t="s">
         <v>27</v>
       </c>
-      <c r="E10" s="11" t="s">
+      <c r="E10" s="12" t="s">
         <v>28</v>
       </c>
-      <c r="F10" s="13">
+      <c r="F10" s="14">
         <v>23.2</v>
       </c>
-      <c r="G10" s="30"/>
-      <c r="H10" s="30"/>
-    </row>
-    <row r="11" ht="75" spans="1:8">
-      <c r="A11" s="10"/>
-      <c r="B11" s="11"/>
-      <c r="C11" s="11" t="s">
+      <c r="G10" s="31"/>
+      <c r="H10" s="31"/>
+    </row>
+    <row r="11" ht="72" spans="1:8">
+      <c r="A11" s="11"/>
+      <c r="B11" s="12"/>
+      <c r="C11" s="12" t="s">
         <v>29</v>
       </c>
-      <c r="D11" s="12" t="s">
+      <c r="D11" s="13" t="s">
         <v>30</v>
       </c>
-      <c r="E11" s="11" t="s">
+      <c r="E11" s="12" t="s">
         <v>31</v>
       </c>
-      <c r="F11" s="13">
+      <c r="F11" s="14">
         <v>16.2</v>
       </c>
-      <c r="G11" s="30"/>
-      <c r="H11" s="30"/>
-    </row>
-    <row r="12" ht="37.5" spans="1:8">
-      <c r="A12" s="10"/>
-      <c r="B12" s="11"/>
-      <c r="C12" s="11"/>
-      <c r="D12" s="12" t="s">
+      <c r="G11" s="31"/>
+      <c r="H11" s="31"/>
+    </row>
+    <row r="12" ht="36" spans="1:8">
+      <c r="A12" s="11"/>
+      <c r="B12" s="12"/>
+      <c r="C12" s="12"/>
+      <c r="D12" s="13" t="s">
         <v>30</v>
       </c>
-      <c r="E12" s="11" t="s">
+      <c r="E12" s="12" t="s">
         <v>32</v>
       </c>
-      <c r="F12" s="13">
+      <c r="F12" s="14">
         <v>16.5</v>
       </c>
-      <c r="G12" s="30"/>
-      <c r="H12" s="30"/>
-    </row>
-    <row r="13" ht="37.5" spans="1:8">
-      <c r="A13" s="10"/>
-      <c r="B13" s="11"/>
-      <c r="C13" s="11"/>
-      <c r="D13" s="12" t="s">
+      <c r="G12" s="31"/>
+      <c r="H12" s="31"/>
+    </row>
+    <row r="13" ht="36" spans="1:8">
+      <c r="A13" s="11"/>
+      <c r="B13" s="12"/>
+      <c r="C13" s="12"/>
+      <c r="D13" s="13" t="s">
         <v>30</v>
       </c>
-      <c r="E13" s="11" t="s">
+      <c r="E13" s="12" t="s">
         <v>33</v>
       </c>
-      <c r="F13" s="13">
+      <c r="F13" s="14">
         <v>16.1</v>
       </c>
-      <c r="G13" s="30"/>
-      <c r="H13" s="30"/>
-    </row>
-    <row r="14" ht="56.25" spans="1:8">
-      <c r="A14" s="31">
+      <c r="G13" s="31"/>
+      <c r="H13" s="31"/>
+    </row>
+    <row r="14" ht="54" spans="1:8">
+      <c r="A14" s="32">
         <v>3</v>
       </c>
-      <c r="B14" s="11" t="s">
+      <c r="B14" s="12" t="s">
         <v>34</v>
       </c>
-      <c r="C14" s="11"/>
-      <c r="D14" s="11" t="s">
+      <c r="C14" s="12"/>
+      <c r="D14" s="12" t="s">
         <v>9</v>
       </c>
-      <c r="E14" s="11" t="s">
+      <c r="E14" s="12" t="s">
         <v>35</v>
       </c>
-      <c r="F14" s="13">
+      <c r="F14" s="14">
         <v>7.4</v>
       </c>
-      <c r="G14" s="30"/>
-      <c r="H14" s="30"/>
-    </row>
-    <row r="15" ht="37.5" spans="1:8">
-      <c r="A15" s="32"/>
-      <c r="B15" s="11"/>
-      <c r="C15" s="11"/>
-      <c r="D15" s="11" t="s">
+      <c r="G14" s="31"/>
+      <c r="H14" s="31"/>
+    </row>
+    <row r="15" ht="36" spans="1:8">
+      <c r="A15" s="33"/>
+      <c r="B15" s="12"/>
+      <c r="C15" s="12"/>
+      <c r="D15" s="12" t="s">
         <v>9</v>
       </c>
-      <c r="E15" s="11" t="s">
+      <c r="E15" s="12" t="s">
         <v>36</v>
       </c>
-      <c r="F15" s="13">
+      <c r="F15" s="14">
         <v>7.5</v>
       </c>
-      <c r="G15" s="30"/>
-      <c r="H15" s="30"/>
-    </row>
-    <row r="16" ht="37.5" spans="1:8">
-      <c r="A16" s="31">
+      <c r="G15" s="31"/>
+      <c r="H15" s="31"/>
+    </row>
+    <row r="16" ht="36" spans="1:8">
+      <c r="A16" s="32">
         <v>4</v>
       </c>
-      <c r="B16" s="11" t="s">
+      <c r="B16" s="12" t="s">
         <v>37</v>
       </c>
-      <c r="C16" s="11"/>
-      <c r="D16" s="11" t="s">
+      <c r="C16" s="12"/>
+      <c r="D16" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="E16" s="11" t="s">
+      <c r="E16" s="12" t="s">
         <v>38</v>
       </c>
-      <c r="F16" s="13">
+      <c r="F16" s="14">
         <v>19.3</v>
       </c>
-      <c r="G16" s="30"/>
-      <c r="H16" s="30"/>
-    </row>
-    <row r="17" ht="37.5" spans="1:8">
-      <c r="A17" s="33"/>
-      <c r="B17" s="11"/>
-      <c r="C17" s="11"/>
-      <c r="D17" s="11" t="s">
+      <c r="G16" s="31"/>
+      <c r="H16" s="31"/>
+    </row>
+    <row r="17" ht="36" spans="1:8">
+      <c r="A17" s="34"/>
+      <c r="B17" s="12"/>
+      <c r="C17" s="12"/>
+      <c r="D17" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="E17" s="11" t="s">
+      <c r="E17" s="12" t="s">
         <v>39</v>
       </c>
-      <c r="F17" s="13">
+      <c r="F17" s="14">
         <v>19.9</v>
       </c>
-      <c r="G17" s="30"/>
-      <c r="H17" s="30"/>
-    </row>
-    <row r="18" ht="37.5" spans="1:8">
-      <c r="A18" s="32"/>
-      <c r="B18" s="11"/>
-      <c r="C18" s="11"/>
-      <c r="D18" s="11" t="s">
+      <c r="G17" s="31"/>
+      <c r="H17" s="31"/>
+    </row>
+    <row r="18" ht="36" spans="1:8">
+      <c r="A18" s="33"/>
+      <c r="B18" s="12"/>
+      <c r="C18" s="12"/>
+      <c r="D18" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="E18" s="11" t="s">
+      <c r="E18" s="12" t="s">
         <v>40</v>
       </c>
-      <c r="F18" s="13">
+      <c r="F18" s="14">
         <v>19.1</v>
       </c>
-      <c r="G18" s="30"/>
-      <c r="H18" s="30"/>
-    </row>
-    <row r="19" ht="37.5" spans="1:8">
-      <c r="A19" s="10">
+      <c r="G18" s="31"/>
+      <c r="H18" s="31"/>
+    </row>
+    <row r="19" ht="36" spans="1:8">
+      <c r="A19" s="11">
         <v>5</v>
       </c>
-      <c r="B19" s="11" t="s">
+      <c r="B19" s="12" t="s">
         <v>41</v>
       </c>
-      <c r="C19" s="11"/>
-      <c r="D19" s="11" t="s">
+      <c r="C19" s="12"/>
+      <c r="D19" s="12" t="s">
         <v>42</v>
       </c>
-      <c r="E19" s="11" t="s">
+      <c r="E19" s="12" t="s">
         <v>43</v>
       </c>
-      <c r="F19" s="13">
+      <c r="F19" s="14">
         <v>15.1</v>
       </c>
-      <c r="G19" s="30"/>
-      <c r="H19" s="30"/>
-    </row>
-    <row r="20" ht="18.75" spans="1:8">
-      <c r="A20" s="10">
+      <c r="G19" s="31"/>
+      <c r="H19" s="31"/>
+    </row>
+    <row r="20" ht="18" spans="1:8">
+      <c r="A20" s="11">
         <v>6</v>
       </c>
-      <c r="B20" s="11" t="s">
+      <c r="B20" s="12" t="s">
         <v>44</v>
       </c>
-      <c r="C20" s="11" t="s">
+      <c r="C20" s="12" t="s">
         <v>45</v>
       </c>
-      <c r="D20" s="11" t="s">
+      <c r="D20" s="12" t="s">
         <v>46</v>
       </c>
-      <c r="E20" s="11"/>
-      <c r="F20" s="13"/>
-      <c r="G20" s="30"/>
-      <c r="H20" s="30"/>
-    </row>
-    <row r="21" ht="18.75" spans="1:8">
-      <c r="A21" s="10"/>
-      <c r="B21" s="11"/>
-      <c r="C21" s="11" t="s">
+      <c r="E20" s="12"/>
+      <c r="F20" s="14"/>
+      <c r="G20" s="31"/>
+      <c r="H20" s="31"/>
+    </row>
+    <row r="21" ht="18" spans="1:8">
+      <c r="A21" s="11"/>
+      <c r="B21" s="12"/>
+      <c r="C21" s="12" t="s">
         <v>47</v>
       </c>
-      <c r="D21" s="11" t="s">
+      <c r="D21" s="12" t="s">
         <v>48</v>
       </c>
-      <c r="E21" s="11"/>
-      <c r="F21" s="13"/>
-      <c r="G21" s="30"/>
-      <c r="H21" s="30"/>
-    </row>
-    <row r="22" ht="18.75" spans="1:8">
-      <c r="A22" s="10"/>
-      <c r="B22" s="11"/>
-      <c r="C22" s="11" t="s">
+      <c r="E21" s="12"/>
+      <c r="F21" s="14"/>
+      <c r="G21" s="31"/>
+      <c r="H21" s="31"/>
+    </row>
+    <row r="22" ht="18" spans="1:8">
+      <c r="A22" s="11"/>
+      <c r="B22" s="12"/>
+      <c r="C22" s="12" t="s">
         <v>49</v>
       </c>
-      <c r="D22" s="11" t="s">
+      <c r="D22" s="12" t="s">
         <v>50</v>
       </c>
-      <c r="E22" s="11"/>
-      <c r="F22" s="13"/>
-      <c r="G22" s="30"/>
-      <c r="H22" s="30"/>
-    </row>
-    <row r="23" ht="18.75" spans="1:8">
-      <c r="A23" s="10"/>
-      <c r="B23" s="11"/>
-      <c r="C23" s="11"/>
-      <c r="D23" s="11" t="s">
+      <c r="E22" s="12"/>
+      <c r="F22" s="14"/>
+      <c r="G22" s="31"/>
+      <c r="H22" s="31"/>
+    </row>
+    <row r="23" ht="18" spans="1:8">
+      <c r="A23" s="11"/>
+      <c r="B23" s="12"/>
+      <c r="C23" s="12"/>
+      <c r="D23" s="12" t="s">
         <v>51</v>
       </c>
-      <c r="E23" s="11"/>
-      <c r="F23" s="13"/>
-      <c r="G23" s="30"/>
-      <c r="H23" s="30"/>
-    </row>
-    <row r="24" ht="37.5" spans="1:8">
-      <c r="A24" s="10"/>
-      <c r="B24" s="11"/>
-      <c r="C24" s="11" t="s">
+      <c r="E23" s="12"/>
+      <c r="F23" s="14"/>
+      <c r="G23" s="31"/>
+      <c r="H23" s="31"/>
+    </row>
+    <row r="24" ht="36" spans="1:8">
+      <c r="A24" s="11"/>
+      <c r="B24" s="12"/>
+      <c r="C24" s="12" t="s">
         <v>52</v>
       </c>
-      <c r="D24" s="11" t="s">
+      <c r="D24" s="12" t="s">
         <v>53</v>
       </c>
-      <c r="E24" s="11"/>
-      <c r="F24" s="13"/>
-      <c r="G24" s="30"/>
-      <c r="H24" s="30"/>
+      <c r="E24" s="12"/>
+      <c r="F24" s="14"/>
+      <c r="G24" s="31"/>
+      <c r="H24" s="31"/>
     </row>
   </sheetData>
   <mergeCells count="16">
@@ -2537,1401 +2576,1563 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:L45"/>
-  <sheetFormatPr defaultColWidth="8.88571428571429" defaultRowHeight="15"/>
+  <dimension ref="A1:N45"/>
+  <sheetFormatPr defaultColWidth="8.88888888888889" defaultRowHeight="14.4"/>
   <cols>
-    <col min="1" max="1" width="7.31428571428571" customWidth="1"/>
-    <col min="2" max="2" width="36.447619047619" customWidth="1"/>
-    <col min="3" max="3" width="25.4952380952381" customWidth="1"/>
-    <col min="4" max="4" width="26.0190476190476" customWidth="1"/>
-    <col min="5" max="5" width="19.7047619047619" style="1" customWidth="1"/>
+    <col min="1" max="1" width="7.31481481481481" customWidth="1"/>
+    <col min="2" max="2" width="36.4444444444444" customWidth="1"/>
+    <col min="3" max="3" width="25.4907407407407" customWidth="1"/>
+    <col min="4" max="4" width="26.0185185185185" customWidth="1"/>
+    <col min="5" max="5" width="19.7037037037037" style="1" customWidth="1"/>
     <col min="6" max="6" width="29.3333333333333" customWidth="1"/>
-    <col min="7" max="7" width="11.1047619047619" style="1" customWidth="1"/>
-    <col min="8" max="8" width="28.4" customWidth="1"/>
-    <col min="9" max="9" width="36.1904761904762" style="2" customWidth="1"/>
-    <col min="10" max="10" width="39.2" style="2" customWidth="1"/>
-    <col min="11" max="11" width="21.8952380952381" style="2" customWidth="1"/>
+    <col min="7" max="7" width="11.1018518518519" style="1" customWidth="1"/>
+    <col min="8" max="8" width="28.3981481481481" customWidth="1"/>
+    <col min="9" max="9" width="36.1944444444444" style="2" customWidth="1"/>
+    <col min="10" max="10" width="39.2037037037037" style="2" customWidth="1"/>
+    <col min="11" max="11" width="21.8981481481481" style="3" customWidth="1"/>
+    <col min="12" max="12" width="38.9907407407407" customWidth="1"/>
+    <col min="13" max="13" width="36.1574074074074" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="18.75" spans="1:11">
-      <c r="A1" s="3" t="s">
+    <row r="1" ht="17.4" spans="1:11">
+      <c r="A1" s="4" t="s">
         <v>54</v>
       </c>
-      <c r="B1" s="4"/>
-      <c r="C1" s="4"/>
-      <c r="D1" s="4"/>
-      <c r="E1" s="4"/>
-      <c r="F1" s="4"/>
-      <c r="G1" s="4"/>
-      <c r="H1" s="5"/>
-      <c r="I1" s="15" t="s">
+      <c r="B1" s="5"/>
+      <c r="C1" s="5"/>
+      <c r="D1" s="5"/>
+      <c r="E1" s="5"/>
+      <c r="F1" s="5"/>
+      <c r="G1" s="5"/>
+      <c r="H1" s="6"/>
+      <c r="I1" s="16" t="s">
         <v>55</v>
       </c>
-      <c r="J1" s="16"/>
-      <c r="K1" s="17"/>
-    </row>
-    <row r="2" ht="37.5" spans="1:11">
-      <c r="A2" s="6" t="s">
+      <c r="J1" s="17"/>
+      <c r="K1" s="18"/>
+    </row>
+    <row r="2" ht="17.4" spans="1:11">
+      <c r="A2" s="7" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="6" t="s">
+      <c r="B2" s="7" t="s">
         <v>56</v>
       </c>
-      <c r="C2" s="6" t="s">
+      <c r="C2" s="7" t="s">
         <v>2</v>
       </c>
-      <c r="D2" s="6" t="s">
+      <c r="D2" s="7" t="s">
         <v>3</v>
       </c>
-      <c r="E2" s="6" t="s">
+      <c r="E2" s="7" t="s">
         <v>57</v>
       </c>
-      <c r="F2" s="6" t="s">
+      <c r="F2" s="7" t="s">
         <v>58</v>
       </c>
-      <c r="G2" s="6" t="s">
+      <c r="G2" s="7" t="s">
         <v>59</v>
       </c>
-      <c r="H2" s="6" t="s">
+      <c r="H2" s="7" t="s">
         <v>60</v>
       </c>
-      <c r="I2" s="18" t="s">
+      <c r="I2" s="19" t="s">
         <v>61</v>
       </c>
-      <c r="J2" s="18" t="s">
+      <c r="J2" s="19" t="s">
         <v>62</v>
       </c>
-      <c r="K2" s="18" t="s">
+      <c r="K2" s="19" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="3" ht="18.75" spans="1:11">
-      <c r="A3" s="7" t="s">
+    <row r="3" ht="18" spans="1:13">
+      <c r="A3" s="8" t="s">
         <v>63</v>
       </c>
-      <c r="B3" s="8"/>
-      <c r="C3" s="8"/>
-      <c r="D3" s="8"/>
-      <c r="E3" s="8"/>
-      <c r="F3" s="8"/>
-      <c r="G3" s="8"/>
-      <c r="H3" s="9"/>
-      <c r="I3" s="19"/>
-      <c r="J3" s="20"/>
-      <c r="K3" s="21"/>
-    </row>
-    <row r="4" ht="112.5" spans="1:11">
-      <c r="A4" s="10">
+      <c r="B3" s="9"/>
+      <c r="C3" s="9"/>
+      <c r="D3" s="9"/>
+      <c r="E3" s="9"/>
+      <c r="F3" s="9"/>
+      <c r="G3" s="9"/>
+      <c r="H3" s="10"/>
+      <c r="I3" s="20"/>
+      <c r="J3" s="21"/>
+      <c r="K3" s="22"/>
+      <c r="L3" t="s">
+        <v>64</v>
+      </c>
+      <c r="M3" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="4" ht="108" spans="1:12">
+      <c r="A4" s="11">
         <v>1</v>
       </c>
-      <c r="B4" s="11" t="s">
-        <v>64</v>
-      </c>
-      <c r="C4" s="11" t="s">
+      <c r="B4" s="12" t="s">
+        <v>66</v>
+      </c>
+      <c r="C4" s="12" t="s">
         <v>9</v>
       </c>
-      <c r="D4" s="11" t="s">
+      <c r="D4" s="12" t="s">
         <v>10</v>
       </c>
-      <c r="E4" s="10">
+      <c r="E4" s="11">
         <v>7.1</v>
       </c>
-      <c r="F4" s="12" t="s">
-        <v>65</v>
-      </c>
-      <c r="G4" s="10" t="s">
-        <v>66</v>
-      </c>
-      <c r="H4" s="12" t="s">
+      <c r="F4" s="13" t="s">
+        <v>67</v>
+      </c>
+      <c r="G4" s="11" t="s">
+        <v>68</v>
+      </c>
+      <c r="H4" s="13" t="s">
         <v>7</v>
       </c>
-      <c r="I4" s="12" t="s">
+      <c r="I4" s="13" t="s">
+        <v>69</v>
+      </c>
+      <c r="J4" s="13" t="s">
+        <v>70</v>
+      </c>
+      <c r="K4" s="11"/>
+      <c r="L4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" ht="234" spans="1:12">
+      <c r="A5" s="11">
+        <v>2</v>
+      </c>
+      <c r="B5" s="13" t="s">
+        <v>71</v>
+      </c>
+      <c r="C5" s="12" t="s">
+        <v>9</v>
+      </c>
+      <c r="D5" s="12" t="s">
+        <v>10</v>
+      </c>
+      <c r="E5" s="11">
+        <v>7.1</v>
+      </c>
+      <c r="F5" s="13" t="s">
         <v>67</v>
       </c>
-      <c r="J4" s="12" t="s">
+      <c r="G5" s="11" t="s">
         <v>68</v>
       </c>
-      <c r="K4" s="12"/>
-    </row>
-    <row r="5" ht="243.75" spans="1:11">
-      <c r="A5" s="10">
-        <v>2</v>
-      </c>
-      <c r="B5" s="12" t="s">
-        <v>69</v>
-      </c>
-      <c r="C5" s="11" t="s">
+      <c r="H5" s="13" t="s">
+        <v>7</v>
+      </c>
+      <c r="I5" s="13" t="s">
+        <v>72</v>
+      </c>
+      <c r="J5" s="13" t="s">
+        <v>73</v>
+      </c>
+      <c r="K5" s="11"/>
+      <c r="L5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" ht="90" spans="1:12">
+      <c r="A6" s="11">
+        <v>3</v>
+      </c>
+      <c r="B6" s="13" t="s">
+        <v>74</v>
+      </c>
+      <c r="C6" s="12" t="s">
         <v>9</v>
       </c>
-      <c r="D5" s="11" t="s">
+      <c r="D6" s="12" t="s">
         <v>10</v>
       </c>
-      <c r="E5" s="10">
+      <c r="E6" s="11">
         <v>7.1</v>
       </c>
-      <c r="F5" s="12" t="s">
-        <v>65</v>
-      </c>
-      <c r="G5" s="10" t="s">
-        <v>66</v>
-      </c>
-      <c r="H5" s="12" t="s">
+      <c r="F6" s="13" t="s">
+        <v>75</v>
+      </c>
+      <c r="G6" s="11" t="s">
+        <v>68</v>
+      </c>
+      <c r="H6" s="13" t="s">
         <v>7</v>
       </c>
-      <c r="I5" s="12" t="s">
-        <v>70</v>
-      </c>
-      <c r="J5" s="12" t="s">
-        <v>71</v>
-      </c>
-      <c r="K5" s="12"/>
-    </row>
-    <row r="6" ht="93.75" spans="1:11">
-      <c r="A6" s="10">
-        <v>3</v>
-      </c>
-      <c r="B6" s="12" t="s">
-        <v>72</v>
-      </c>
-      <c r="C6" s="11" t="s">
+      <c r="I6" s="13" t="s">
+        <v>76</v>
+      </c>
+      <c r="J6" s="13" t="s">
+        <v>73</v>
+      </c>
+      <c r="K6" s="11"/>
+      <c r="L6">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" ht="108" spans="1:14">
+      <c r="A7" s="11">
+        <v>4</v>
+      </c>
+      <c r="B7" s="13" t="s">
+        <v>77</v>
+      </c>
+      <c r="C7" s="12" t="s">
+        <v>12</v>
+      </c>
+      <c r="D7" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="E7" s="14">
+        <v>19.8</v>
+      </c>
+      <c r="F7" s="13" t="s">
+        <v>67</v>
+      </c>
+      <c r="G7" s="11" t="s">
+        <v>68</v>
+      </c>
+      <c r="H7" s="13" t="s">
+        <v>7</v>
+      </c>
+      <c r="I7" s="13" t="s">
+        <v>78</v>
+      </c>
+      <c r="J7" s="13" t="s">
+        <v>79</v>
+      </c>
+      <c r="K7" s="11" t="s">
+        <v>80</v>
+      </c>
+      <c r="L7">
+        <v>1</v>
+      </c>
+      <c r="M7" t="s">
+        <v>81</v>
+      </c>
+      <c r="N7" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="8" ht="72" spans="1:13">
+      <c r="A8" s="11">
+        <v>5</v>
+      </c>
+      <c r="B8" s="13" t="s">
+        <v>83</v>
+      </c>
+      <c r="C8" s="12" t="s">
+        <v>12</v>
+      </c>
+      <c r="D8" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="E8" s="14">
+        <v>19.8</v>
+      </c>
+      <c r="F8" s="13" t="s">
+        <v>84</v>
+      </c>
+      <c r="G8" s="11" t="s">
+        <v>68</v>
+      </c>
+      <c r="H8" s="13" t="s">
+        <v>7</v>
+      </c>
+      <c r="I8" s="13" t="s">
+        <v>85</v>
+      </c>
+      <c r="J8" s="13" t="s">
+        <v>86</v>
+      </c>
+      <c r="K8" s="11" t="s">
+        <v>80</v>
+      </c>
+      <c r="L8">
+        <v>1</v>
+      </c>
+      <c r="M8" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="9" ht="108" spans="1:12">
+      <c r="A9" s="11">
+        <v>6</v>
+      </c>
+      <c r="B9" s="12" t="s">
+        <v>87</v>
+      </c>
+      <c r="C9" s="13" t="s">
+        <v>15</v>
+      </c>
+      <c r="D9" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="E9" s="14">
+        <v>12.1</v>
+      </c>
+      <c r="F9" s="13" t="s">
+        <v>84</v>
+      </c>
+      <c r="G9" s="11" t="s">
+        <v>68</v>
+      </c>
+      <c r="H9" s="13" t="s">
+        <v>7</v>
+      </c>
+      <c r="I9" s="13" t="s">
+        <v>88</v>
+      </c>
+      <c r="J9" s="13" t="s">
+        <v>89</v>
+      </c>
+      <c r="K9" s="11" t="s">
+        <v>80</v>
+      </c>
+      <c r="L9" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="10" ht="108" spans="1:12">
+      <c r="A10" s="11">
+        <v>7</v>
+      </c>
+      <c r="B10" s="12" t="s">
+        <v>91</v>
+      </c>
+      <c r="C10" s="13" t="s">
+        <v>15</v>
+      </c>
+      <c r="D10" s="12" t="s">
+        <v>17</v>
+      </c>
+      <c r="E10" s="14">
+        <v>12.2</v>
+      </c>
+      <c r="F10" s="13" t="s">
+        <v>84</v>
+      </c>
+      <c r="G10" s="11" t="s">
+        <v>68</v>
+      </c>
+      <c r="H10" s="13" t="s">
+        <v>7</v>
+      </c>
+      <c r="I10" s="13" t="s">
+        <v>92</v>
+      </c>
+      <c r="J10" s="13" t="s">
+        <v>93</v>
+      </c>
+      <c r="K10" s="11" t="s">
+        <v>80</v>
+      </c>
+      <c r="L10" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="11" ht="108" spans="1:13">
+      <c r="A11" s="11">
+        <v>8</v>
+      </c>
+      <c r="B11" s="12" t="s">
+        <v>94</v>
+      </c>
+      <c r="C11" s="13" t="s">
+        <v>15</v>
+      </c>
+      <c r="D11" s="12" t="s">
+        <v>95</v>
+      </c>
+      <c r="E11" s="14" t="s">
+        <v>96</v>
+      </c>
+      <c r="F11" s="13" t="s">
+        <v>84</v>
+      </c>
+      <c r="G11" s="11" t="s">
+        <v>68</v>
+      </c>
+      <c r="H11" s="13" t="s">
+        <v>7</v>
+      </c>
+      <c r="I11" s="13" t="s">
+        <v>97</v>
+      </c>
+      <c r="J11" s="13" t="s">
+        <v>98</v>
+      </c>
+      <c r="K11" s="11"/>
+      <c r="L11">
+        <v>1</v>
+      </c>
+      <c r="M11" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="12" ht="90" spans="1:12">
+      <c r="A12" s="11">
         <v>9</v>
       </c>
-      <c r="D6" s="11" t="s">
+      <c r="B12" s="13" t="s">
+        <v>100</v>
+      </c>
+      <c r="C12" s="12" t="s">
+        <v>18</v>
+      </c>
+      <c r="D12" s="12" t="s">
+        <v>19</v>
+      </c>
+      <c r="E12" s="14">
+        <v>8.3</v>
+      </c>
+      <c r="F12" s="13" t="s">
+        <v>84</v>
+      </c>
+      <c r="G12" s="11" t="s">
+        <v>101</v>
+      </c>
+      <c r="H12" s="13" t="s">
+        <v>7</v>
+      </c>
+      <c r="I12" s="13" t="s">
+        <v>102</v>
+      </c>
+      <c r="J12" s="13" t="s">
+        <v>103</v>
+      </c>
+      <c r="K12" s="11" t="s">
+        <v>80</v>
+      </c>
+      <c r="L12">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13" ht="108" spans="1:12">
+      <c r="A13" s="11">
         <v>10</v>
       </c>
-      <c r="E6" s="10">
+      <c r="B13" s="13" t="s">
+        <v>104</v>
+      </c>
+      <c r="C13" s="12" t="s">
+        <v>18</v>
+      </c>
+      <c r="D13" s="12" t="s">
+        <v>19</v>
+      </c>
+      <c r="E13" s="14">
+        <v>8.3</v>
+      </c>
+      <c r="F13" s="13" t="s">
+        <v>84</v>
+      </c>
+      <c r="G13" s="11" t="s">
+        <v>101</v>
+      </c>
+      <c r="H13" s="13" t="s">
+        <v>7</v>
+      </c>
+      <c r="I13" s="13" t="s">
+        <v>105</v>
+      </c>
+      <c r="J13" s="13" t="s">
+        <v>106</v>
+      </c>
+      <c r="K13" s="11" t="s">
+        <v>80</v>
+      </c>
+      <c r="L13">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14" ht="108" spans="1:12">
+      <c r="A14" s="11">
+        <v>11</v>
+      </c>
+      <c r="B14" s="13" t="s">
+        <v>107</v>
+      </c>
+      <c r="C14" s="12" t="s">
+        <v>18</v>
+      </c>
+      <c r="D14" s="12" t="s">
+        <v>25</v>
+      </c>
+      <c r="E14" s="14">
+        <v>8.2</v>
+      </c>
+      <c r="F14" s="13" t="s">
+        <v>84</v>
+      </c>
+      <c r="G14" s="11" t="s">
+        <v>101</v>
+      </c>
+      <c r="H14" s="13" t="s">
+        <v>23</v>
+      </c>
+      <c r="I14" s="13" t="s">
+        <v>108</v>
+      </c>
+      <c r="J14" s="13" t="s">
+        <v>109</v>
+      </c>
+      <c r="K14" s="11"/>
+      <c r="L14">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" ht="18" spans="1:11">
+      <c r="A15" s="15" t="s">
+        <v>110</v>
+      </c>
+      <c r="B15" s="15"/>
+      <c r="C15" s="15"/>
+      <c r="D15" s="15"/>
+      <c r="E15" s="15"/>
+      <c r="F15" s="15"/>
+      <c r="G15" s="15"/>
+      <c r="H15" s="15"/>
+      <c r="I15" s="23"/>
+      <c r="J15" s="24"/>
+      <c r="K15" s="25"/>
+    </row>
+    <row r="16" ht="108" spans="1:12">
+      <c r="A16" s="11">
+        <v>12</v>
+      </c>
+      <c r="B16" s="13" t="s">
+        <v>111</v>
+      </c>
+      <c r="C16" s="12" t="s">
+        <v>9</v>
+      </c>
+      <c r="D16" s="12" t="s">
+        <v>10</v>
+      </c>
+      <c r="E16" s="11">
         <v>7.1</v>
       </c>
-      <c r="F6" s="12" t="s">
-        <v>73</v>
-      </c>
-      <c r="G6" s="10" t="s">
-        <v>66</v>
-      </c>
-      <c r="H6" s="12" t="s">
+      <c r="F16" s="13" t="s">
+        <v>112</v>
+      </c>
+      <c r="G16" s="11" t="s">
+        <v>101</v>
+      </c>
+      <c r="H16" s="13" t="s">
         <v>7</v>
       </c>
-      <c r="I6" s="12" t="s">
-        <v>74</v>
-      </c>
-      <c r="J6" s="12" t="s">
-        <v>71</v>
-      </c>
-      <c r="K6" s="12"/>
-    </row>
-    <row r="7" ht="112.5" spans="1:11">
-      <c r="A7" s="10">
-        <v>4</v>
-      </c>
-      <c r="B7" s="12" t="s">
+      <c r="I16" s="13" t="s">
+        <v>113</v>
+      </c>
+      <c r="J16" s="13" t="s">
+        <v>114</v>
+      </c>
+      <c r="K16" s="11"/>
+      <c r="L16" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17" ht="72" spans="1:12">
+      <c r="A17" s="11">
+        <v>13</v>
+      </c>
+      <c r="B17" s="13" t="s">
+        <v>115</v>
+      </c>
+      <c r="C17" s="12" t="s">
+        <v>9</v>
+      </c>
+      <c r="D17" s="12" t="s">
+        <v>10</v>
+      </c>
+      <c r="E17" s="11">
+        <v>7.1</v>
+      </c>
+      <c r="F17" s="13" t="s">
+        <v>84</v>
+      </c>
+      <c r="G17" s="11" t="s">
+        <v>101</v>
+      </c>
+      <c r="H17" s="13" t="s">
+        <v>7</v>
+      </c>
+      <c r="I17" s="13" t="s">
+        <v>116</v>
+      </c>
+      <c r="J17" s="13" t="s">
+        <v>117</v>
+      </c>
+      <c r="K17" s="11"/>
+      <c r="L17" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18" ht="72" spans="1:12">
+      <c r="A18" s="11">
+        <v>14</v>
+      </c>
+      <c r="B18" s="13" t="s">
+        <v>118</v>
+      </c>
+      <c r="C18" s="12" t="s">
+        <v>9</v>
+      </c>
+      <c r="D18" s="12" t="s">
+        <v>10</v>
+      </c>
+      <c r="E18" s="11">
+        <v>7.1</v>
+      </c>
+      <c r="F18" s="13" t="s">
+        <v>119</v>
+      </c>
+      <c r="G18" s="11" t="s">
+        <v>101</v>
+      </c>
+      <c r="H18" s="13" t="s">
+        <v>7</v>
+      </c>
+      <c r="I18" s="13" t="s">
+        <v>120</v>
+      </c>
+      <c r="J18" s="13" t="s">
+        <v>121</v>
+      </c>
+      <c r="K18" s="11"/>
+      <c r="L18" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19" ht="108" spans="1:13">
+      <c r="A19" s="11">
+        <v>15</v>
+      </c>
+      <c r="B19" s="13" t="s">
+        <v>122</v>
+      </c>
+      <c r="C19" s="12" t="s">
+        <v>12</v>
+      </c>
+      <c r="D19" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="E19" s="14">
+        <v>19.8</v>
+      </c>
+      <c r="F19" s="13" t="s">
+        <v>112</v>
+      </c>
+      <c r="G19" s="11" t="s">
+        <v>68</v>
+      </c>
+      <c r="H19" s="13" t="s">
+        <v>7</v>
+      </c>
+      <c r="I19" s="13" t="s">
+        <v>123</v>
+      </c>
+      <c r="J19" s="13" t="s">
+        <v>124</v>
+      </c>
+      <c r="K19" s="11"/>
+      <c r="L19" s="2" t="s">
+        <v>125</v>
+      </c>
+      <c r="M19" t="s">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="20" ht="216" spans="1:13">
+      <c r="A20" s="11">
+        <v>16</v>
+      </c>
+      <c r="B20" s="13" t="s">
+        <v>127</v>
+      </c>
+      <c r="C20" s="12" t="s">
+        <v>12</v>
+      </c>
+      <c r="D20" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="E20" s="14">
+        <v>19.8</v>
+      </c>
+      <c r="F20" s="13" t="s">
+        <v>119</v>
+      </c>
+      <c r="G20" s="11" t="s">
+        <v>68</v>
+      </c>
+      <c r="H20" s="13" t="s">
+        <v>7</v>
+      </c>
+      <c r="I20" s="13" t="s">
+        <v>128</v>
+      </c>
+      <c r="J20" s="13" t="s">
+        <v>129</v>
+      </c>
+      <c r="K20" s="11" t="s">
+        <v>80</v>
+      </c>
+      <c r="L20" s="2">
+        <v>1</v>
+      </c>
+      <c r="M20" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="21" ht="108" spans="1:12">
+      <c r="A21" s="11">
+        <v>17</v>
+      </c>
+      <c r="B21" s="13" t="s">
+        <v>131</v>
+      </c>
+      <c r="C21" s="13" t="s">
+        <v>15</v>
+      </c>
+      <c r="D21" s="12" t="s">
+        <v>95</v>
+      </c>
+      <c r="E21" s="14" t="s">
+        <v>96</v>
+      </c>
+      <c r="F21" s="13" t="s">
+        <v>84</v>
+      </c>
+      <c r="G21" s="11" t="s">
+        <v>68</v>
+      </c>
+      <c r="H21" s="13" t="s">
+        <v>7</v>
+      </c>
+      <c r="I21" s="13" t="s">
+        <v>132</v>
+      </c>
+      <c r="J21" s="13" t="s">
+        <v>98</v>
+      </c>
+      <c r="K21" s="11" t="s">
+        <v>80</v>
+      </c>
+      <c r="L21" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="22" ht="108" spans="1:12">
+      <c r="A22" s="11">
+        <v>18</v>
+      </c>
+      <c r="B22" s="13" t="s">
+        <v>133</v>
+      </c>
+      <c r="C22" s="12" t="s">
+        <v>18</v>
+      </c>
+      <c r="D22" s="12" t="s">
+        <v>25</v>
+      </c>
+      <c r="E22" s="14">
+        <v>8.2</v>
+      </c>
+      <c r="F22" s="13" t="s">
+        <v>84</v>
+      </c>
+      <c r="G22" s="11" t="s">
+        <v>101</v>
+      </c>
+      <c r="H22" s="13" t="s">
+        <v>23</v>
+      </c>
+      <c r="I22" s="13" t="s">
+        <v>134</v>
+      </c>
+      <c r="J22" s="13" t="s">
+        <v>98</v>
+      </c>
+      <c r="K22" s="11"/>
+      <c r="L22" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23" ht="180" spans="1:12">
+      <c r="A23" s="11">
+        <v>19</v>
+      </c>
+      <c r="B23" s="13" t="s">
+        <v>135</v>
+      </c>
+      <c r="C23" s="13" t="s">
+        <v>30</v>
+      </c>
+      <c r="D23" s="12" t="s">
+        <v>136</v>
+      </c>
+      <c r="E23" s="11" t="s">
+        <v>137</v>
+      </c>
+      <c r="F23" s="13" t="s">
+        <v>138</v>
+      </c>
+      <c r="G23" s="11" t="s">
+        <v>101</v>
+      </c>
+      <c r="H23" s="13" t="s">
+        <v>23</v>
+      </c>
+      <c r="I23" s="13"/>
+      <c r="J23" s="13" t="s">
+        <v>139</v>
+      </c>
+      <c r="K23" s="11"/>
+      <c r="L23" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24" ht="72" spans="1:12">
+      <c r="A24" s="11">
+        <v>20</v>
+      </c>
+      <c r="B24" s="13" t="s">
+        <v>140</v>
+      </c>
+      <c r="C24" s="13" t="s">
+        <v>30</v>
+      </c>
+      <c r="D24" s="12" t="s">
+        <v>33</v>
+      </c>
+      <c r="E24" s="14">
+        <v>16.1</v>
+      </c>
+      <c r="F24" s="13" t="s">
+        <v>67</v>
+      </c>
+      <c r="G24" s="11" t="s">
+        <v>101</v>
+      </c>
+      <c r="H24" s="13" t="s">
+        <v>23</v>
+      </c>
+      <c r="I24" s="13"/>
+      <c r="J24" s="13" t="s">
+        <v>139</v>
+      </c>
+      <c r="K24" s="11"/>
+      <c r="L24" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25" ht="90" spans="1:12">
+      <c r="A25" s="11">
+        <v>21</v>
+      </c>
+      <c r="B25" s="13" t="s">
+        <v>141</v>
+      </c>
+      <c r="C25" s="12" t="s">
+        <v>9</v>
+      </c>
+      <c r="D25" s="12" t="s">
+        <v>142</v>
+      </c>
+      <c r="E25" s="14">
+        <v>7.4</v>
+      </c>
+      <c r="F25" s="13" t="s">
+        <v>84</v>
+      </c>
+      <c r="G25" s="11" t="s">
+        <v>101</v>
+      </c>
+      <c r="H25" s="13" t="s">
+        <v>34</v>
+      </c>
+      <c r="I25" s="13" t="s">
+        <v>143</v>
+      </c>
+      <c r="J25" s="13" t="s">
+        <v>144</v>
+      </c>
+      <c r="K25" s="11"/>
+      <c r="L25" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26" ht="72" spans="1:13">
+      <c r="A26" s="11">
+        <v>22</v>
+      </c>
+      <c r="B26" s="13" t="s">
+        <v>145</v>
+      </c>
+      <c r="C26" s="12" t="s">
+        <v>9</v>
+      </c>
+      <c r="D26" s="12" t="s">
+        <v>36</v>
+      </c>
+      <c r="E26" s="14">
+        <v>7.5</v>
+      </c>
+      <c r="F26" s="13" t="s">
+        <v>67</v>
+      </c>
+      <c r="G26" s="11" t="s">
+        <v>101</v>
+      </c>
+      <c r="H26" s="13" t="s">
+        <v>34</v>
+      </c>
+      <c r="I26" s="13" t="s">
+        <v>146</v>
+      </c>
+      <c r="J26" s="13" t="s">
+        <v>147</v>
+      </c>
+      <c r="K26" s="11"/>
+      <c r="L26" s="2">
+        <v>0</v>
+      </c>
+      <c r="M26" t="s">
+        <v>148</v>
+      </c>
+    </row>
+    <row r="27" ht="72" spans="1:12">
+      <c r="A27" s="11">
+        <v>23</v>
+      </c>
+      <c r="B27" s="13" t="s">
+        <v>149</v>
+      </c>
+      <c r="C27" s="12" t="s">
+        <v>9</v>
+      </c>
+      <c r="D27" s="12" t="s">
+        <v>36</v>
+      </c>
+      <c r="E27" s="14">
+        <v>7.5</v>
+      </c>
+      <c r="F27" s="13" t="s">
         <v>75</v>
       </c>
-      <c r="C7" s="11" t="s">
+      <c r="G27" s="11" t="s">
+        <v>101</v>
+      </c>
+      <c r="H27" s="13" t="s">
+        <v>34</v>
+      </c>
+      <c r="I27" s="13" t="s">
+        <v>150</v>
+      </c>
+      <c r="J27" s="13" t="s">
+        <v>147</v>
+      </c>
+      <c r="K27" s="11" t="s">
+        <v>80</v>
+      </c>
+      <c r="L27" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="28" ht="72" spans="1:12">
+      <c r="A28" s="11">
+        <v>24</v>
+      </c>
+      <c r="B28" s="13" t="s">
+        <v>151</v>
+      </c>
+      <c r="C28" s="12" t="s">
+        <v>9</v>
+      </c>
+      <c r="D28" s="12" t="s">
+        <v>36</v>
+      </c>
+      <c r="E28" s="14">
+        <v>7.5</v>
+      </c>
+      <c r="F28" s="13" t="s">
+        <v>119</v>
+      </c>
+      <c r="G28" s="11" t="s">
+        <v>101</v>
+      </c>
+      <c r="H28" s="13" t="s">
+        <v>34</v>
+      </c>
+      <c r="I28" s="13" t="s">
+        <v>152</v>
+      </c>
+      <c r="J28" s="13" t="s">
+        <v>147</v>
+      </c>
+      <c r="K28" s="11" t="s">
+        <v>80</v>
+      </c>
+      <c r="L28" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="29" ht="72" spans="1:12">
+      <c r="A29" s="11">
+        <v>25</v>
+      </c>
+      <c r="B29" s="13" t="s">
+        <v>153</v>
+      </c>
+      <c r="C29" s="12" t="s">
+        <v>9</v>
+      </c>
+      <c r="D29" s="12" t="s">
+        <v>36</v>
+      </c>
+      <c r="E29" s="14">
+        <v>7.5</v>
+      </c>
+      <c r="F29" s="13" t="s">
+        <v>112</v>
+      </c>
+      <c r="G29" s="11" t="s">
+        <v>101</v>
+      </c>
+      <c r="H29" s="13" t="s">
+        <v>34</v>
+      </c>
+      <c r="I29" s="13" t="s">
+        <v>154</v>
+      </c>
+      <c r="J29" s="13" t="s">
+        <v>155</v>
+      </c>
+      <c r="K29" s="11"/>
+      <c r="L29" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="30" ht="108" spans="1:12">
+      <c r="A30" s="11">
+        <v>26</v>
+      </c>
+      <c r="B30" s="13" t="s">
+        <v>156</v>
+      </c>
+      <c r="C30" s="12" t="s">
+        <v>9</v>
+      </c>
+      <c r="D30" s="12" t="s">
+        <v>36</v>
+      </c>
+      <c r="E30" s="14">
+        <v>7.5</v>
+      </c>
+      <c r="F30" s="13" t="s">
+        <v>84</v>
+      </c>
+      <c r="G30" s="11" t="s">
+        <v>101</v>
+      </c>
+      <c r="H30" s="13" t="s">
+        <v>34</v>
+      </c>
+      <c r="I30" s="13" t="s">
+        <v>157</v>
+      </c>
+      <c r="J30" s="13" t="s">
+        <v>158</v>
+      </c>
+      <c r="K30" s="11"/>
+      <c r="L30" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="31" ht="90" spans="1:12">
+      <c r="A31" s="11">
+        <v>27</v>
+      </c>
+      <c r="B31" s="13" t="s">
+        <v>159</v>
+      </c>
+      <c r="C31" s="12" t="s">
+        <v>27</v>
+      </c>
+      <c r="D31" s="12" t="s">
+        <v>28</v>
+      </c>
+      <c r="E31" s="14">
+        <v>23.2</v>
+      </c>
+      <c r="F31" s="13" t="s">
+        <v>84</v>
+      </c>
+      <c r="G31" s="11" t="s">
+        <v>101</v>
+      </c>
+      <c r="H31" s="13" t="s">
+        <v>23</v>
+      </c>
+      <c r="I31" s="13" t="s">
+        <v>160</v>
+      </c>
+      <c r="J31" s="13" t="s">
+        <v>161</v>
+      </c>
+      <c r="K31" s="11"/>
+      <c r="L31" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="32" ht="72" spans="1:12">
+      <c r="A32" s="11">
+        <v>28</v>
+      </c>
+      <c r="B32" s="13" t="s">
+        <v>162</v>
+      </c>
+      <c r="C32" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="D7" s="11" t="s">
-        <v>13</v>
-      </c>
-      <c r="E7" s="13">
-        <v>19.8</v>
-      </c>
-      <c r="F7" s="12" t="s">
-        <v>65</v>
-      </c>
-      <c r="G7" s="10" t="s">
-        <v>66</v>
-      </c>
-      <c r="H7" s="12" t="s">
+      <c r="D32" s="12" t="s">
+        <v>39</v>
+      </c>
+      <c r="E32" s="14">
+        <v>19.9</v>
+      </c>
+      <c r="F32" s="13" t="s">
+        <v>67</v>
+      </c>
+      <c r="G32" s="11" t="s">
+        <v>68</v>
+      </c>
+      <c r="H32" s="13" t="s">
+        <v>37</v>
+      </c>
+      <c r="I32" s="13" t="s">
+        <v>163</v>
+      </c>
+      <c r="J32" s="13" t="s">
+        <v>164</v>
+      </c>
+      <c r="K32" s="11"/>
+      <c r="L32" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="33" ht="54" spans="1:12">
+      <c r="A33" s="11">
+        <v>29</v>
+      </c>
+      <c r="B33" s="13" t="s">
+        <v>165</v>
+      </c>
+      <c r="C33" s="12" t="s">
+        <v>12</v>
+      </c>
+      <c r="D33" s="12" t="s">
+        <v>39</v>
+      </c>
+      <c r="E33" s="14">
+        <v>19.9</v>
+      </c>
+      <c r="F33" s="13" t="s">
+        <v>84</v>
+      </c>
+      <c r="G33" s="11" t="s">
+        <v>68</v>
+      </c>
+      <c r="H33" s="13" t="s">
+        <v>37</v>
+      </c>
+      <c r="I33" s="13" t="s">
+        <v>166</v>
+      </c>
+      <c r="J33" s="13" t="s">
+        <v>167</v>
+      </c>
+      <c r="K33" s="11"/>
+      <c r="L33" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="34" ht="90" spans="1:12">
+      <c r="A34" s="11">
+        <v>30</v>
+      </c>
+      <c r="B34" s="13" t="s">
+        <v>168</v>
+      </c>
+      <c r="C34" s="12" t="s">
+        <v>12</v>
+      </c>
+      <c r="D34" s="12" t="s">
+        <v>40</v>
+      </c>
+      <c r="E34" s="14">
+        <v>19.1</v>
+      </c>
+      <c r="F34" s="13" t="s">
+        <v>84</v>
+      </c>
+      <c r="G34" s="11" t="s">
+        <v>68</v>
+      </c>
+      <c r="H34" s="13" t="s">
+        <v>37</v>
+      </c>
+      <c r="I34" s="13" t="s">
+        <v>169</v>
+      </c>
+      <c r="J34" s="13" t="s">
+        <v>170</v>
+      </c>
+      <c r="K34" s="11"/>
+      <c r="L34" s="2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="35" ht="54" spans="1:13">
+      <c r="A35" s="11">
+        <v>31</v>
+      </c>
+      <c r="B35" s="13" t="s">
+        <v>171</v>
+      </c>
+      <c r="C35" s="12" t="s">
+        <v>42</v>
+      </c>
+      <c r="D35" s="12" t="s">
+        <v>43</v>
+      </c>
+      <c r="E35" s="14">
+        <v>15.1</v>
+      </c>
+      <c r="F35" s="13" t="s">
+        <v>84</v>
+      </c>
+      <c r="G35" s="11" t="s">
+        <v>172</v>
+      </c>
+      <c r="H35" s="13" t="s">
+        <v>41</v>
+      </c>
+      <c r="I35" s="13" t="s">
+        <v>173</v>
+      </c>
+      <c r="J35" s="13" t="s">
+        <v>174</v>
+      </c>
+      <c r="K35" s="11" t="s">
+        <v>80</v>
+      </c>
+      <c r="L35" s="2">
+        <v>1</v>
+      </c>
+      <c r="M35">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="36" ht="18" spans="1:12">
+      <c r="A36" s="15" t="s">
+        <v>175</v>
+      </c>
+      <c r="B36" s="15"/>
+      <c r="C36" s="15"/>
+      <c r="D36" s="15"/>
+      <c r="E36" s="15"/>
+      <c r="F36" s="15"/>
+      <c r="G36" s="15"/>
+      <c r="H36" s="15"/>
+      <c r="I36" s="26"/>
+      <c r="J36" s="27"/>
+      <c r="K36" s="28"/>
+      <c r="L36" s="2"/>
+    </row>
+    <row r="37" ht="54" spans="1:12">
+      <c r="A37" s="11">
+        <v>32</v>
+      </c>
+      <c r="B37" s="13" t="s">
+        <v>176</v>
+      </c>
+      <c r="C37" s="12"/>
+      <c r="D37" s="12"/>
+      <c r="E37" s="14"/>
+      <c r="F37" s="13" t="s">
+        <v>177</v>
+      </c>
+      <c r="G37" s="11" t="s">
+        <v>68</v>
+      </c>
+      <c r="H37" s="13" t="s">
         <v>7</v>
       </c>
-      <c r="I7" s="12" t="s">
-        <v>76</v>
-      </c>
-      <c r="J7" s="12" t="s">
-        <v>77</v>
-      </c>
-      <c r="K7" s="12"/>
-    </row>
-    <row r="8" ht="75" spans="1:11">
-      <c r="A8" s="10">
-        <v>5</v>
-      </c>
-      <c r="B8" s="12" t="s">
-        <v>78</v>
-      </c>
-      <c r="C8" s="11" t="s">
-        <v>12</v>
-      </c>
-      <c r="D8" s="11" t="s">
-        <v>13</v>
-      </c>
-      <c r="E8" s="13">
-        <v>19.8</v>
-      </c>
-      <c r="F8" s="12" t="s">
-        <v>79</v>
-      </c>
-      <c r="G8" s="10" t="s">
-        <v>66</v>
-      </c>
-      <c r="H8" s="12" t="s">
+      <c r="I37" s="13" t="s">
+        <v>178</v>
+      </c>
+      <c r="J37" s="13" t="s">
+        <v>179</v>
+      </c>
+      <c r="K37" s="11" t="s">
+        <v>80</v>
+      </c>
+      <c r="L37">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="38" ht="54" spans="1:12">
+      <c r="A38" s="11">
+        <v>33</v>
+      </c>
+      <c r="B38" s="13" t="s">
+        <v>180</v>
+      </c>
+      <c r="C38" s="12"/>
+      <c r="D38" s="12"/>
+      <c r="E38" s="14"/>
+      <c r="F38" s="13" t="s">
+        <v>177</v>
+      </c>
+      <c r="G38" s="11" t="s">
+        <v>68</v>
+      </c>
+      <c r="H38" s="13" t="s">
         <v>7</v>
       </c>
-      <c r="I8" s="12" t="s">
+      <c r="I38" s="13" t="s">
+        <v>181</v>
+      </c>
+      <c r="J38" s="13" t="s">
+        <v>179</v>
+      </c>
+      <c r="K38" s="11" t="s">
         <v>80</v>
       </c>
-      <c r="J8" s="12" t="s">
-        <v>81</v>
-      </c>
-      <c r="K8" s="12"/>
-    </row>
-    <row r="9" ht="112.5" spans="1:11">
-      <c r="A9" s="10">
-        <v>6</v>
-      </c>
-      <c r="B9" s="11" t="s">
-        <v>82</v>
-      </c>
-      <c r="C9" s="12" t="s">
-        <v>15</v>
-      </c>
-      <c r="D9" s="11" t="s">
-        <v>16</v>
-      </c>
-      <c r="E9" s="13">
-        <v>12.1</v>
-      </c>
-      <c r="F9" s="12" t="s">
-        <v>79</v>
-      </c>
-      <c r="G9" s="10" t="s">
-        <v>66</v>
-      </c>
-      <c r="H9" s="12" t="s">
+      <c r="L38">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="39" ht="79" customHeight="1" spans="1:12">
+      <c r="A39" s="11">
+        <v>34</v>
+      </c>
+      <c r="B39" s="13" t="s">
+        <v>182</v>
+      </c>
+      <c r="C39" s="12"/>
+      <c r="D39" s="12"/>
+      <c r="E39" s="14"/>
+      <c r="F39" s="13" t="s">
+        <v>177</v>
+      </c>
+      <c r="G39" s="11" t="s">
+        <v>68</v>
+      </c>
+      <c r="H39" s="13" t="s">
         <v>7</v>
       </c>
-      <c r="I9" s="12" t="s">
-        <v>83</v>
-      </c>
-      <c r="J9" s="12" t="s">
-        <v>84</v>
-      </c>
-      <c r="K9" s="12"/>
-    </row>
-    <row r="10" ht="112.5" spans="1:11">
-      <c r="A10" s="10">
+      <c r="I39" s="13" t="s">
+        <v>183</v>
+      </c>
+      <c r="J39" s="13" t="s">
+        <v>179</v>
+      </c>
+      <c r="K39" s="11" t="s">
+        <v>80</v>
+      </c>
+      <c r="L39">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="40" ht="54" spans="1:12">
+      <c r="A40" s="11">
+        <v>35</v>
+      </c>
+      <c r="B40" s="13" t="s">
+        <v>184</v>
+      </c>
+      <c r="C40" s="12"/>
+      <c r="D40" s="12"/>
+      <c r="E40" s="14"/>
+      <c r="F40" s="13" t="s">
+        <v>177</v>
+      </c>
+      <c r="G40" s="11" t="s">
+        <v>68</v>
+      </c>
+      <c r="H40" s="13" t="s">
         <v>7</v>
       </c>
-      <c r="B10" s="11" t="s">
-        <v>85</v>
-      </c>
-      <c r="C10" s="12" t="s">
-        <v>15</v>
-      </c>
-      <c r="D10" s="11" t="s">
-        <v>17</v>
-      </c>
-      <c r="E10" s="13">
-        <v>12.2</v>
-      </c>
-      <c r="F10" s="12" t="s">
-        <v>79</v>
-      </c>
-      <c r="G10" s="10" t="s">
-        <v>66</v>
-      </c>
-      <c r="H10" s="12" t="s">
+      <c r="I40" s="13" t="s">
+        <v>185</v>
+      </c>
+      <c r="J40" s="13" t="s">
+        <v>186</v>
+      </c>
+      <c r="K40" s="11"/>
+      <c r="L40" t="s">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="41" ht="36" spans="1:12">
+      <c r="A41" s="11">
+        <v>36</v>
+      </c>
+      <c r="B41" s="13" t="s">
+        <v>188</v>
+      </c>
+      <c r="C41" s="12"/>
+      <c r="D41" s="12"/>
+      <c r="E41" s="14"/>
+      <c r="F41" s="13" t="s">
+        <v>177</v>
+      </c>
+      <c r="G41" s="11" t="s">
+        <v>68</v>
+      </c>
+      <c r="H41" s="13" t="s">
         <v>7</v>
       </c>
-      <c r="I10" s="12" t="s">
-        <v>86</v>
-      </c>
-      <c r="J10" s="12" t="s">
-        <v>87</v>
-      </c>
-      <c r="K10" s="12"/>
-    </row>
-    <row r="11" ht="112.5" spans="1:11">
-      <c r="A11" s="10">
-        <v>8</v>
-      </c>
-      <c r="B11" s="11" t="s">
-        <v>88</v>
-      </c>
-      <c r="C11" s="12" t="s">
-        <v>15</v>
-      </c>
-      <c r="D11" s="11" t="s">
-        <v>89</v>
-      </c>
-      <c r="E11" s="13" t="s">
-        <v>90</v>
-      </c>
-      <c r="F11" s="12" t="s">
-        <v>79</v>
-      </c>
-      <c r="G11" s="10" t="s">
-        <v>66</v>
-      </c>
-      <c r="H11" s="12" t="s">
+      <c r="I41" s="13" t="s">
+        <v>189</v>
+      </c>
+      <c r="J41" s="13" t="s">
+        <v>190</v>
+      </c>
+      <c r="K41" s="11" t="s">
+        <v>80</v>
+      </c>
+      <c r="L41">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="42" ht="54" spans="1:12">
+      <c r="A42" s="11">
+        <v>37</v>
+      </c>
+      <c r="B42" s="13" t="s">
+        <v>191</v>
+      </c>
+      <c r="C42" s="12"/>
+      <c r="D42" s="12"/>
+      <c r="E42" s="14"/>
+      <c r="F42" s="13" t="s">
+        <v>177</v>
+      </c>
+      <c r="G42" s="11" t="s">
+        <v>68</v>
+      </c>
+      <c r="H42" s="13" t="s">
         <v>7</v>
       </c>
-      <c r="I11" s="12" t="s">
-        <v>91</v>
-      </c>
-      <c r="J11" s="12" t="s">
-        <v>92</v>
-      </c>
-      <c r="K11" s="12"/>
-    </row>
-    <row r="12" ht="93.75" spans="1:11">
-      <c r="A12" s="10">
-        <v>9</v>
-      </c>
-      <c r="B12" s="12" t="s">
-        <v>93</v>
-      </c>
-      <c r="C12" s="11" t="s">
-        <v>18</v>
-      </c>
-      <c r="D12" s="11" t="s">
-        <v>19</v>
-      </c>
-      <c r="E12" s="13">
-        <v>8.3</v>
-      </c>
-      <c r="F12" s="12" t="s">
-        <v>79</v>
-      </c>
-      <c r="G12" s="10" t="s">
-        <v>94</v>
-      </c>
-      <c r="H12" s="12" t="s">
+      <c r="I42" s="13" t="s">
+        <v>192</v>
+      </c>
+      <c r="J42" s="13" t="s">
+        <v>193</v>
+      </c>
+      <c r="K42" s="11"/>
+      <c r="L42">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="43" ht="54" spans="1:12">
+      <c r="A43" s="11">
+        <v>38</v>
+      </c>
+      <c r="B43" s="13" t="s">
+        <v>194</v>
+      </c>
+      <c r="C43" s="12"/>
+      <c r="D43" s="12"/>
+      <c r="E43" s="14"/>
+      <c r="F43" s="13" t="s">
+        <v>177</v>
+      </c>
+      <c r="G43" s="11" t="s">
+        <v>68</v>
+      </c>
+      <c r="H43" s="13" t="s">
         <v>7</v>
       </c>
-      <c r="I12" s="12" t="s">
-        <v>95</v>
-      </c>
-      <c r="J12" s="12" t="s">
-        <v>96</v>
-      </c>
-      <c r="K12" s="12"/>
-    </row>
-    <row r="13" ht="112.5" spans="1:11">
-      <c r="A13" s="10">
-        <v>10</v>
-      </c>
-      <c r="B13" s="12" t="s">
-        <v>97</v>
-      </c>
-      <c r="C13" s="11" t="s">
-        <v>18</v>
-      </c>
-      <c r="D13" s="11" t="s">
-        <v>19</v>
-      </c>
-      <c r="E13" s="13">
-        <v>8.3</v>
-      </c>
-      <c r="F13" s="12" t="s">
-        <v>79</v>
-      </c>
-      <c r="G13" s="10" t="s">
-        <v>94</v>
-      </c>
-      <c r="H13" s="12" t="s">
+      <c r="I43" s="13" t="s">
+        <v>195</v>
+      </c>
+      <c r="J43" s="13" t="s">
+        <v>193</v>
+      </c>
+      <c r="K43" s="11"/>
+      <c r="L43">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="44" ht="72" spans="1:12">
+      <c r="A44" s="11">
+        <v>39</v>
+      </c>
+      <c r="B44" s="13" t="s">
+        <v>196</v>
+      </c>
+      <c r="C44" s="12"/>
+      <c r="D44" s="12"/>
+      <c r="E44" s="14"/>
+      <c r="F44" s="13" t="s">
+        <v>177</v>
+      </c>
+      <c r="G44" s="11" t="s">
+        <v>68</v>
+      </c>
+      <c r="H44" s="13" t="s">
         <v>7</v>
       </c>
-      <c r="I13" s="12" t="s">
-        <v>98</v>
-      </c>
-      <c r="J13" s="12" t="s">
-        <v>99</v>
-      </c>
-      <c r="K13" s="12"/>
-    </row>
-    <row r="14" ht="112.5" spans="1:11">
-      <c r="A14" s="10">
-        <v>11</v>
-      </c>
-      <c r="B14" s="12" t="s">
-        <v>100</v>
-      </c>
-      <c r="C14" s="11" t="s">
-        <v>18</v>
-      </c>
-      <c r="D14" s="11" t="s">
-        <v>25</v>
-      </c>
-      <c r="E14" s="13">
-        <v>8.2</v>
-      </c>
-      <c r="F14" s="12" t="s">
-        <v>79</v>
-      </c>
-      <c r="G14" s="10" t="s">
-        <v>94</v>
-      </c>
-      <c r="H14" s="12" t="s">
-        <v>23</v>
-      </c>
-      <c r="I14" s="12" t="s">
-        <v>101</v>
-      </c>
-      <c r="J14" s="12" t="s">
-        <v>102</v>
-      </c>
-      <c r="K14" s="12"/>
-    </row>
-    <row r="15" ht="18.75" spans="1:11">
-      <c r="A15" s="14" t="s">
-        <v>103</v>
-      </c>
-      <c r="B15" s="14"/>
-      <c r="C15" s="14"/>
-      <c r="D15" s="14"/>
-      <c r="E15" s="14"/>
-      <c r="F15" s="14"/>
-      <c r="G15" s="14"/>
-      <c r="H15" s="14"/>
-      <c r="I15" s="22"/>
-      <c r="J15" s="23"/>
-      <c r="K15" s="24"/>
-    </row>
-    <row r="16" ht="112.5" spans="1:12">
-      <c r="A16" s="10">
-        <v>12</v>
-      </c>
-      <c r="B16" s="12" t="s">
-        <v>104</v>
-      </c>
-      <c r="C16" s="11" t="s">
-        <v>9</v>
-      </c>
-      <c r="D16" s="11" t="s">
-        <v>10</v>
-      </c>
-      <c r="E16" s="10">
-        <v>7.1</v>
-      </c>
-      <c r="F16" s="12" t="s">
-        <v>105</v>
-      </c>
-      <c r="G16" s="10" t="s">
-        <v>94</v>
-      </c>
-      <c r="H16" s="12" t="s">
+      <c r="I44" s="13" t="s">
+        <v>197</v>
+      </c>
+      <c r="J44" s="13" t="s">
+        <v>198</v>
+      </c>
+      <c r="K44" s="11"/>
+      <c r="L44">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="45" ht="54" spans="1:12">
+      <c r="A45" s="11">
+        <v>40</v>
+      </c>
+      <c r="B45" s="13" t="s">
+        <v>199</v>
+      </c>
+      <c r="C45" s="12"/>
+      <c r="D45" s="12"/>
+      <c r="E45" s="14"/>
+      <c r="F45" s="13" t="s">
+        <v>177</v>
+      </c>
+      <c r="G45" s="11" t="s">
+        <v>68</v>
+      </c>
+      <c r="H45" s="13" t="s">
         <v>7</v>
       </c>
-      <c r="I16" s="12" t="s">
-        <v>106</v>
-      </c>
-      <c r="J16" s="12" t="s">
-        <v>107</v>
-      </c>
-      <c r="K16" s="12"/>
-      <c r="L16" s="2"/>
-    </row>
-    <row r="17" ht="75" spans="1:12">
-      <c r="A17" s="10">
-        <v>13</v>
-      </c>
-      <c r="B17" s="12" t="s">
-        <v>108</v>
-      </c>
-      <c r="C17" s="11" t="s">
-        <v>9</v>
-      </c>
-      <c r="D17" s="11" t="s">
-        <v>10</v>
-      </c>
-      <c r="E17" s="10">
-        <v>7.1</v>
-      </c>
-      <c r="F17" s="12" t="s">
-        <v>79</v>
-      </c>
-      <c r="G17" s="10" t="s">
-        <v>94</v>
-      </c>
-      <c r="H17" s="12" t="s">
-        <v>7</v>
-      </c>
-      <c r="I17" s="12" t="s">
-        <v>109</v>
-      </c>
-      <c r="J17" s="12" t="s">
-        <v>110</v>
-      </c>
-      <c r="K17" s="12"/>
-      <c r="L17" s="2"/>
-    </row>
-    <row r="18" ht="75" spans="1:12">
-      <c r="A18" s="10">
-        <v>14</v>
-      </c>
-      <c r="B18" s="12" t="s">
-        <v>111</v>
-      </c>
-      <c r="C18" s="11" t="s">
-        <v>9</v>
-      </c>
-      <c r="D18" s="11" t="s">
-        <v>10</v>
-      </c>
-      <c r="E18" s="10">
-        <v>7.1</v>
-      </c>
-      <c r="F18" s="12" t="s">
-        <v>112</v>
-      </c>
-      <c r="G18" s="10" t="s">
-        <v>94</v>
-      </c>
-      <c r="H18" s="12" t="s">
-        <v>7</v>
-      </c>
-      <c r="I18" s="12" t="s">
-        <v>113</v>
-      </c>
-      <c r="J18" s="12" t="s">
-        <v>114</v>
-      </c>
-      <c r="K18" s="12"/>
-      <c r="L18" s="2"/>
-    </row>
-    <row r="19" ht="112.5" spans="1:12">
-      <c r="A19" s="10">
-        <v>15</v>
-      </c>
-      <c r="B19" s="12" t="s">
-        <v>115</v>
-      </c>
-      <c r="C19" s="11" t="s">
-        <v>12</v>
-      </c>
-      <c r="D19" s="11" t="s">
-        <v>13</v>
-      </c>
-      <c r="E19" s="13">
-        <v>19.8</v>
-      </c>
-      <c r="F19" s="12" t="s">
-        <v>105</v>
-      </c>
-      <c r="G19" s="10" t="s">
-        <v>66</v>
-      </c>
-      <c r="H19" s="12" t="s">
-        <v>7</v>
-      </c>
-      <c r="I19" s="12" t="s">
-        <v>116</v>
-      </c>
-      <c r="J19" s="12" t="s">
-        <v>117</v>
-      </c>
-      <c r="K19" s="12"/>
-      <c r="L19" s="2"/>
-    </row>
-    <row r="20" ht="225" spans="1:12">
-      <c r="A20" s="10">
-        <v>16</v>
-      </c>
-      <c r="B20" s="12" t="s">
-        <v>118</v>
-      </c>
-      <c r="C20" s="11" t="s">
-        <v>12</v>
-      </c>
-      <c r="D20" s="11" t="s">
-        <v>13</v>
-      </c>
-      <c r="E20" s="13">
-        <v>19.8</v>
-      </c>
-      <c r="F20" s="12" t="s">
-        <v>112</v>
-      </c>
-      <c r="G20" s="10" t="s">
-        <v>66</v>
-      </c>
-      <c r="H20" s="12" t="s">
-        <v>7</v>
-      </c>
-      <c r="I20" s="12" t="s">
-        <v>119</v>
-      </c>
-      <c r="J20" s="12" t="s">
-        <v>120</v>
-      </c>
-      <c r="K20" s="12"/>
-      <c r="L20" s="2"/>
-    </row>
-    <row r="21" ht="112.5" spans="1:12">
-      <c r="A21" s="10">
-        <v>17</v>
-      </c>
-      <c r="B21" s="12" t="s">
-        <v>121</v>
-      </c>
-      <c r="C21" s="12" t="s">
-        <v>15</v>
-      </c>
-      <c r="D21" s="11" t="s">
-        <v>89</v>
-      </c>
-      <c r="E21" s="13" t="s">
-        <v>90</v>
-      </c>
-      <c r="F21" s="12" t="s">
-        <v>79</v>
-      </c>
-      <c r="G21" s="10" t="s">
-        <v>66</v>
-      </c>
-      <c r="H21" s="12" t="s">
-        <v>7</v>
-      </c>
-      <c r="I21" s="12" t="s">
-        <v>122</v>
-      </c>
-      <c r="J21" s="12" t="s">
-        <v>92</v>
-      </c>
-      <c r="K21" s="12"/>
-      <c r="L21" s="2"/>
-    </row>
-    <row r="22" ht="112.5" spans="1:12">
-      <c r="A22" s="10">
-        <v>18</v>
-      </c>
-      <c r="B22" s="12" t="s">
-        <v>123</v>
-      </c>
-      <c r="C22" s="11" t="s">
-        <v>18</v>
-      </c>
-      <c r="D22" s="11" t="s">
-        <v>25</v>
-      </c>
-      <c r="E22" s="13">
-        <v>8.2</v>
-      </c>
-      <c r="F22" s="12" t="s">
-        <v>79</v>
-      </c>
-      <c r="G22" s="10" t="s">
-        <v>94</v>
-      </c>
-      <c r="H22" s="12" t="s">
-        <v>23</v>
-      </c>
-      <c r="I22" s="12" t="s">
-        <v>124</v>
-      </c>
-      <c r="J22" s="12" t="s">
-        <v>92</v>
-      </c>
-      <c r="K22" s="12"/>
-      <c r="L22" s="2"/>
-    </row>
-    <row r="23" ht="187.5" spans="1:12">
-      <c r="A23" s="10">
-        <v>19</v>
-      </c>
-      <c r="B23" s="12" t="s">
-        <v>125</v>
-      </c>
-      <c r="C23" s="12" t="s">
-        <v>30</v>
-      </c>
-      <c r="D23" s="11" t="s">
-        <v>126</v>
-      </c>
-      <c r="E23" s="10" t="s">
-        <v>127</v>
-      </c>
-      <c r="F23" s="12" t="s">
-        <v>128</v>
-      </c>
-      <c r="G23" s="10" t="s">
-        <v>94</v>
-      </c>
-      <c r="H23" s="12" t="s">
-        <v>23</v>
-      </c>
-      <c r="I23" s="12"/>
-      <c r="J23" s="12" t="s">
-        <v>129</v>
-      </c>
-      <c r="K23" s="12"/>
-      <c r="L23" s="2"/>
-    </row>
-    <row r="24" ht="75" spans="1:12">
-      <c r="A24" s="10">
-        <v>20</v>
-      </c>
-      <c r="B24" s="12" t="s">
-        <v>130</v>
-      </c>
-      <c r="C24" s="12" t="s">
-        <v>30</v>
-      </c>
-      <c r="D24" s="11" t="s">
-        <v>33</v>
-      </c>
-      <c r="E24" s="13">
-        <v>16.1</v>
-      </c>
-      <c r="F24" s="12" t="s">
-        <v>65</v>
-      </c>
-      <c r="G24" s="10" t="s">
-        <v>94</v>
-      </c>
-      <c r="H24" s="12" t="s">
-        <v>23</v>
-      </c>
-      <c r="I24" s="12"/>
-      <c r="J24" s="12" t="s">
-        <v>129</v>
-      </c>
-      <c r="K24" s="12"/>
-      <c r="L24" s="2"/>
-    </row>
-    <row r="25" ht="93.75" spans="1:12">
-      <c r="A25" s="10">
-        <v>21</v>
-      </c>
-      <c r="B25" s="12" t="s">
-        <v>131</v>
-      </c>
-      <c r="C25" s="11" t="s">
-        <v>9</v>
-      </c>
-      <c r="D25" s="11" t="s">
-        <v>132</v>
-      </c>
-      <c r="E25" s="13">
-        <v>7.4</v>
-      </c>
-      <c r="F25" s="12" t="s">
-        <v>79</v>
-      </c>
-      <c r="G25" s="10" t="s">
-        <v>94</v>
-      </c>
-      <c r="H25" s="12" t="s">
-        <v>34</v>
-      </c>
-      <c r="I25" s="12" t="s">
-        <v>133</v>
-      </c>
-      <c r="J25" s="12" t="s">
-        <v>134</v>
-      </c>
-      <c r="K25" s="12"/>
-      <c r="L25" s="2"/>
-    </row>
-    <row r="26" ht="75" spans="1:12">
-      <c r="A26" s="10">
-        <v>22</v>
-      </c>
-      <c r="B26" s="12" t="s">
-        <v>135</v>
-      </c>
-      <c r="C26" s="11" t="s">
-        <v>9</v>
-      </c>
-      <c r="D26" s="11" t="s">
-        <v>36</v>
-      </c>
-      <c r="E26" s="13">
-        <v>7.5</v>
-      </c>
-      <c r="F26" s="12" t="s">
-        <v>65</v>
-      </c>
-      <c r="G26" s="10" t="s">
-        <v>94</v>
-      </c>
-      <c r="H26" s="12" t="s">
-        <v>34</v>
-      </c>
-      <c r="I26" s="12" t="s">
-        <v>136</v>
-      </c>
-      <c r="J26" s="12" t="s">
-        <v>137</v>
-      </c>
-      <c r="K26" s="12"/>
-      <c r="L26" s="2"/>
-    </row>
-    <row r="27" ht="75" spans="1:12">
-      <c r="A27" s="10">
-        <v>23</v>
-      </c>
-      <c r="B27" s="12" t="s">
-        <v>138</v>
-      </c>
-      <c r="C27" s="11" t="s">
-        <v>9</v>
-      </c>
-      <c r="D27" s="11" t="s">
-        <v>36</v>
-      </c>
-      <c r="E27" s="13">
-        <v>7.5</v>
-      </c>
-      <c r="F27" s="12" t="s">
-        <v>73</v>
-      </c>
-      <c r="G27" s="10" t="s">
-        <v>94</v>
-      </c>
-      <c r="H27" s="12" t="s">
-        <v>34</v>
-      </c>
-      <c r="I27" s="12" t="s">
-        <v>139</v>
-      </c>
-      <c r="J27" s="12" t="s">
-        <v>137</v>
-      </c>
-      <c r="K27" s="12"/>
-      <c r="L27" s="2"/>
-    </row>
-    <row r="28" ht="75" spans="1:12">
-      <c r="A28" s="10">
-        <v>24</v>
-      </c>
-      <c r="B28" s="12" t="s">
-        <v>140</v>
-      </c>
-      <c r="C28" s="11" t="s">
-        <v>9</v>
-      </c>
-      <c r="D28" s="11" t="s">
-        <v>36</v>
-      </c>
-      <c r="E28" s="13">
-        <v>7.5</v>
-      </c>
-      <c r="F28" s="12" t="s">
-        <v>112</v>
-      </c>
-      <c r="G28" s="10" t="s">
-        <v>94</v>
-      </c>
-      <c r="H28" s="12" t="s">
-        <v>34</v>
-      </c>
-      <c r="I28" s="12" t="s">
-        <v>141</v>
-      </c>
-      <c r="J28" s="12" t="s">
-        <v>137</v>
-      </c>
-      <c r="K28" s="12"/>
-      <c r="L28" s="2"/>
-    </row>
-    <row r="29" ht="75" spans="1:12">
-      <c r="A29" s="10">
-        <v>25</v>
-      </c>
-      <c r="B29" s="12" t="s">
-        <v>142</v>
-      </c>
-      <c r="C29" s="11" t="s">
-        <v>9</v>
-      </c>
-      <c r="D29" s="11" t="s">
-        <v>36</v>
-      </c>
-      <c r="E29" s="13">
-        <v>7.5</v>
-      </c>
-      <c r="F29" s="12" t="s">
-        <v>105</v>
-      </c>
-      <c r="G29" s="10" t="s">
-        <v>94</v>
-      </c>
-      <c r="H29" s="12" t="s">
-        <v>34</v>
-      </c>
-      <c r="I29" s="12" t="s">
-        <v>143</v>
-      </c>
-      <c r="J29" s="12" t="s">
-        <v>144</v>
-      </c>
-      <c r="K29" s="12"/>
-      <c r="L29" s="2"/>
-    </row>
-    <row r="30" ht="112.5" spans="1:12">
-      <c r="A30" s="10">
-        <v>26</v>
-      </c>
-      <c r="B30" s="12" t="s">
-        <v>145</v>
-      </c>
-      <c r="C30" s="11" t="s">
-        <v>9</v>
-      </c>
-      <c r="D30" s="11" t="s">
-        <v>36</v>
-      </c>
-      <c r="E30" s="13">
-        <v>7.5</v>
-      </c>
-      <c r="F30" s="12" t="s">
-        <v>79</v>
-      </c>
-      <c r="G30" s="10" t="s">
-        <v>94</v>
-      </c>
-      <c r="H30" s="12" t="s">
-        <v>34</v>
-      </c>
-      <c r="I30" s="12" t="s">
-        <v>146</v>
-      </c>
-      <c r="J30" s="12" t="s">
-        <v>147</v>
-      </c>
-      <c r="K30" s="12"/>
-      <c r="L30" s="2"/>
-    </row>
-    <row r="31" ht="93.75" spans="1:12">
-      <c r="A31" s="10">
-        <v>27</v>
-      </c>
-      <c r="B31" s="12" t="s">
-        <v>148</v>
-      </c>
-      <c r="C31" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="D31" s="11" t="s">
-        <v>28</v>
-      </c>
-      <c r="E31" s="13">
-        <v>23.2</v>
-      </c>
-      <c r="F31" s="12" t="s">
-        <v>79</v>
-      </c>
-      <c r="G31" s="10" t="s">
-        <v>94</v>
-      </c>
-      <c r="H31" s="12" t="s">
-        <v>23</v>
-      </c>
-      <c r="I31" s="12" t="s">
-        <v>149</v>
-      </c>
-      <c r="J31" s="12" t="s">
-        <v>150</v>
-      </c>
-      <c r="K31" s="12"/>
-      <c r="L31" s="2"/>
-    </row>
-    <row r="32" ht="75" spans="1:12">
-      <c r="A32" s="10">
-        <v>28</v>
-      </c>
-      <c r="B32" s="12" t="s">
-        <v>151</v>
-      </c>
-      <c r="C32" s="11" t="s">
-        <v>12</v>
-      </c>
-      <c r="D32" s="11" t="s">
-        <v>39</v>
-      </c>
-      <c r="E32" s="13">
-        <v>19.9</v>
-      </c>
-      <c r="F32" s="12" t="s">
-        <v>65</v>
-      </c>
-      <c r="G32" s="10" t="s">
-        <v>66</v>
-      </c>
-      <c r="H32" s="12" t="s">
-        <v>37</v>
-      </c>
-      <c r="I32" s="12" t="s">
-        <v>152</v>
-      </c>
-      <c r="J32" s="12" t="s">
-        <v>153</v>
-      </c>
-      <c r="K32" s="12"/>
-      <c r="L32" s="2"/>
-    </row>
-    <row r="33" ht="56.25" spans="1:12">
-      <c r="A33" s="10">
-        <v>29</v>
-      </c>
-      <c r="B33" s="12" t="s">
-        <v>154</v>
-      </c>
-      <c r="C33" s="11" t="s">
-        <v>12</v>
-      </c>
-      <c r="D33" s="11" t="s">
-        <v>39</v>
-      </c>
-      <c r="E33" s="13">
-        <v>19.9</v>
-      </c>
-      <c r="F33" s="12" t="s">
-        <v>79</v>
-      </c>
-      <c r="G33" s="10" t="s">
-        <v>66</v>
-      </c>
-      <c r="H33" s="12" t="s">
-        <v>37</v>
-      </c>
-      <c r="I33" s="12" t="s">
-        <v>155</v>
-      </c>
-      <c r="J33" s="12" t="s">
-        <v>156</v>
-      </c>
-      <c r="K33" s="12"/>
-      <c r="L33" s="2"/>
-    </row>
-    <row r="34" ht="93.75" spans="1:12">
-      <c r="A34" s="10">
-        <v>30</v>
-      </c>
-      <c r="B34" s="12" t="s">
-        <v>157</v>
-      </c>
-      <c r="C34" s="11" t="s">
-        <v>12</v>
-      </c>
-      <c r="D34" s="11" t="s">
-        <v>40</v>
-      </c>
-      <c r="E34" s="13">
-        <v>19.1</v>
-      </c>
-      <c r="F34" s="12" t="s">
-        <v>79</v>
-      </c>
-      <c r="G34" s="10" t="s">
-        <v>66</v>
-      </c>
-      <c r="H34" s="12" t="s">
-        <v>37</v>
-      </c>
-      <c r="I34" s="12" t="s">
-        <v>158</v>
-      </c>
-      <c r="J34" s="12" t="s">
-        <v>159</v>
-      </c>
-      <c r="K34" s="12"/>
-      <c r="L34" s="2"/>
-    </row>
-    <row r="35" ht="56.25" spans="1:12">
-      <c r="A35" s="10">
-        <v>31</v>
-      </c>
-      <c r="B35" s="12" t="s">
-        <v>160</v>
-      </c>
-      <c r="C35" s="11" t="s">
-        <v>42</v>
-      </c>
-      <c r="D35" s="11" t="s">
-        <v>43</v>
-      </c>
-      <c r="E35" s="13">
-        <v>15.1</v>
-      </c>
-      <c r="F35" s="12" t="s">
-        <v>79</v>
-      </c>
-      <c r="G35" s="10" t="s">
-        <v>161</v>
-      </c>
-      <c r="H35" s="12" t="s">
-        <v>41</v>
-      </c>
-      <c r="I35" s="12" t="s">
-        <v>162</v>
-      </c>
-      <c r="J35" s="12" t="s">
-        <v>163</v>
-      </c>
-      <c r="K35" s="12"/>
-      <c r="L35" s="2"/>
-    </row>
-    <row r="36" ht="18.75" spans="1:12">
-      <c r="A36" s="14" t="s">
-        <v>164</v>
-      </c>
-      <c r="B36" s="14"/>
-      <c r="C36" s="14"/>
-      <c r="D36" s="14"/>
-      <c r="E36" s="14"/>
-      <c r="F36" s="14"/>
-      <c r="G36" s="14"/>
-      <c r="H36" s="14"/>
-      <c r="I36" s="25"/>
-      <c r="J36" s="26"/>
-      <c r="K36" s="27"/>
-      <c r="L36" s="2"/>
-    </row>
-    <row r="37" ht="56.25" spans="1:11">
-      <c r="A37" s="10">
-        <v>32</v>
-      </c>
-      <c r="B37" s="12" t="s">
-        <v>165</v>
-      </c>
-      <c r="C37" s="11"/>
-      <c r="D37" s="11"/>
-      <c r="E37" s="13"/>
-      <c r="F37" s="12" t="s">
-        <v>166</v>
-      </c>
-      <c r="G37" s="10" t="s">
-        <v>66</v>
-      </c>
-      <c r="H37" s="12" t="s">
-        <v>7</v>
-      </c>
-      <c r="I37" s="12" t="s">
-        <v>167</v>
-      </c>
-      <c r="J37" s="12" t="s">
-        <v>168</v>
-      </c>
-      <c r="K37" s="12"/>
-    </row>
-    <row r="38" ht="56.25" spans="1:11">
-      <c r="A38" s="10">
-        <v>33</v>
-      </c>
-      <c r="B38" s="12" t="s">
-        <v>169</v>
-      </c>
-      <c r="C38" s="11"/>
-      <c r="D38" s="11"/>
-      <c r="E38" s="13"/>
-      <c r="F38" s="12" t="s">
-        <v>166</v>
-      </c>
-      <c r="G38" s="10" t="s">
-        <v>66</v>
-      </c>
-      <c r="H38" s="12" t="s">
-        <v>7</v>
-      </c>
-      <c r="I38" s="12" t="s">
-        <v>170</v>
-      </c>
-      <c r="J38" s="12" t="s">
-        <v>168</v>
-      </c>
-      <c r="K38" s="12"/>
-    </row>
-    <row r="39" ht="79" customHeight="1" spans="1:11">
-      <c r="A39" s="10">
-        <v>34</v>
-      </c>
-      <c r="B39" s="12" t="s">
-        <v>171</v>
-      </c>
-      <c r="C39" s="11"/>
-      <c r="D39" s="11"/>
-      <c r="E39" s="13"/>
-      <c r="F39" s="12" t="s">
-        <v>166</v>
-      </c>
-      <c r="G39" s="10" t="s">
-        <v>66</v>
-      </c>
-      <c r="H39" s="12" t="s">
-        <v>7</v>
-      </c>
-      <c r="I39" s="12" t="s">
-        <v>172</v>
-      </c>
-      <c r="J39" s="12" t="s">
-        <v>168</v>
-      </c>
-      <c r="K39" s="12"/>
-    </row>
-    <row r="40" ht="56.25" spans="1:11">
-      <c r="A40" s="10">
-        <v>35</v>
-      </c>
-      <c r="B40" s="12" t="s">
-        <v>173</v>
-      </c>
-      <c r="C40" s="11"/>
-      <c r="D40" s="11"/>
-      <c r="E40" s="13"/>
-      <c r="F40" s="12" t="s">
-        <v>166</v>
-      </c>
-      <c r="G40" s="10" t="s">
-        <v>66</v>
-      </c>
-      <c r="H40" s="12" t="s">
-        <v>7</v>
-      </c>
-      <c r="I40" s="12" t="s">
-        <v>174</v>
-      </c>
-      <c r="J40" s="12" t="s">
-        <v>175</v>
-      </c>
-      <c r="K40" s="12"/>
-    </row>
-    <row r="41" ht="37.5" spans="1:11">
-      <c r="A41" s="10">
-        <v>36</v>
-      </c>
-      <c r="B41" s="12" t="s">
-        <v>176</v>
-      </c>
-      <c r="C41" s="11"/>
-      <c r="D41" s="11"/>
-      <c r="E41" s="13"/>
-      <c r="F41" s="12" t="s">
-        <v>166</v>
-      </c>
-      <c r="G41" s="10" t="s">
-        <v>66</v>
-      </c>
-      <c r="H41" s="12" t="s">
-        <v>7</v>
-      </c>
-      <c r="I41" s="12" t="s">
-        <v>177</v>
-      </c>
-      <c r="J41" s="12" t="s">
-        <v>178</v>
-      </c>
-      <c r="K41" s="12"/>
-    </row>
-    <row r="42" ht="56.25" spans="1:11">
-      <c r="A42" s="10">
-        <v>37</v>
-      </c>
-      <c r="B42" s="12" t="s">
-        <v>179</v>
-      </c>
-      <c r="C42" s="11"/>
-      <c r="D42" s="11"/>
-      <c r="E42" s="13"/>
-      <c r="F42" s="12" t="s">
-        <v>166</v>
-      </c>
-      <c r="G42" s="10" t="s">
-        <v>66</v>
-      </c>
-      <c r="H42" s="12" t="s">
-        <v>7</v>
-      </c>
-      <c r="I42" s="12" t="s">
-        <v>180</v>
-      </c>
-      <c r="J42" s="12" t="s">
-        <v>181</v>
-      </c>
-      <c r="K42" s="12"/>
-    </row>
-    <row r="43" ht="56.25" spans="1:11">
-      <c r="A43" s="10">
-        <v>38</v>
-      </c>
-      <c r="B43" s="12" t="s">
-        <v>182</v>
-      </c>
-      <c r="C43" s="11"/>
-      <c r="D43" s="11"/>
-      <c r="E43" s="13"/>
-      <c r="F43" s="12" t="s">
-        <v>166</v>
-      </c>
-      <c r="G43" s="10" t="s">
-        <v>66</v>
-      </c>
-      <c r="H43" s="12" t="s">
-        <v>7</v>
-      </c>
-      <c r="I43" s="12" t="s">
-        <v>183</v>
-      </c>
-      <c r="J43" s="12" t="s">
-        <v>181</v>
-      </c>
-      <c r="K43" s="12"/>
-    </row>
-    <row r="44" ht="75" spans="1:11">
-      <c r="A44" s="10">
-        <v>39</v>
-      </c>
-      <c r="B44" s="12" t="s">
-        <v>184</v>
-      </c>
-      <c r="C44" s="11"/>
-      <c r="D44" s="11"/>
-      <c r="E44" s="13"/>
-      <c r="F44" s="12" t="s">
-        <v>166</v>
-      </c>
-      <c r="G44" s="10" t="s">
-        <v>66</v>
-      </c>
-      <c r="H44" s="12" t="s">
-        <v>7</v>
-      </c>
-      <c r="I44" s="12" t="s">
-        <v>185</v>
-      </c>
-      <c r="J44" s="12" t="s">
-        <v>186</v>
-      </c>
-      <c r="K44" s="12"/>
-    </row>
-    <row r="45" ht="75" spans="1:11">
-      <c r="A45" s="10">
-        <v>40</v>
-      </c>
-      <c r="B45" s="12" t="s">
-        <v>187</v>
-      </c>
-      <c r="C45" s="11"/>
-      <c r="D45" s="11"/>
-      <c r="E45" s="13"/>
-      <c r="F45" s="12" t="s">
-        <v>166</v>
-      </c>
-      <c r="G45" s="10" t="s">
-        <v>66</v>
-      </c>
-      <c r="H45" s="12" t="s">
-        <v>7</v>
-      </c>
-      <c r="I45" s="12" t="s">
-        <v>188</v>
-      </c>
-      <c r="J45" s="12" t="s">
-        <v>189</v>
-      </c>
-      <c r="K45" s="12"/>
+      <c r="I45" s="13" t="s">
+        <v>200</v>
+      </c>
+      <c r="J45" s="13" t="s">
+        <v>201</v>
+      </c>
+      <c r="K45" s="11"/>
+      <c r="L45">
+        <v>0</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="8">

</xml_diff>